<commit_message>
feat(research): 16/08 update — Coppa Italia field data, market U-turns, ops baked
- Rigoristi: Deiola dal campo (Cagliari), Parma senza designato, Zaccagni 1°
  unanime (correzione), Milan di fatto Ramos (Nkunku fuori rosa)
- Mercato: Suzuki->Aston Villa (PSG saltato), Falcone resta al Lecce, Vicario
  raffreddato (Juve su Dibu Martinez), Frattesi/Spence/Obrador ufficiali
- Campo: XI Coppa Italia 14-16/8 (Maldini panchina, Ghedjemis fuori, Kvernadze
  e Fini promossi, Halhal/Hainaut nuovi, Mascardi in porta Toro)
- Infortuni: Maignan e Lautaro recuperati, Tavares e Leao peggiorati, nuovi
  Comuzzo/Casale/Yildiz/Gilmour
- 87 wishlist_ops applicate e baked in asta.xlsx (verifica di equivalenza);
  listone.xlsx aggiornato dall'utente (7 nuovi listati, cambi squadra)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asta.xlsx
+++ b/asta.xlsx
@@ -624,7 +624,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -724,7 +724,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -824,7 +824,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -915,7 +915,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -948,7 +948,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="it-IT"/>
         </a:p>
@@ -1103,7 +1103,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="it-IT"/>
                 </a:p>
@@ -1132,7 +1132,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="it-IT"/>
                 </a:p>
@@ -1161,7 +1161,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="it-IT"/>
                 </a:p>
@@ -1190,7 +1190,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="it-IT"/>
                 </a:p>
@@ -1219,7 +1219,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -1309,7 +1309,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="it-IT"/>
         </a:p>
@@ -1425,7 +1425,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -1660,7 +1660,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -1751,7 +1751,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -1784,7 +1784,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="it-IT"/>
         </a:p>
@@ -1897,7 +1897,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -2123,7 +2123,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="it-IT"/>
               </a:p>
@@ -2274,7 +2274,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -2365,7 +2365,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="it-IT"/>
           </a:p>
@@ -2398,7 +2398,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="it-IT"/>
         </a:p>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="F10" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Rientrato (55-60%)</t>
         </is>
       </c>
       <c r="G10" s="35" t="inlineStr">
@@ -4362,11 +4362,11 @@
         </is>
       </c>
       <c r="I10" s="10" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="J10" s="36" t="inlineStr">
         <is>
-          <t>Rientra dal Mondiale solo il 16/8: TORRIANI favorito (~65%) alla 1ª. Bio social ripulita ma il club lo blinda. Non pagarlo pensando all'avvio.</t>
+          <t>RIENTRATO IN ANTICIPO (15/8): favorito 55-60% su Torriani per la 1ª, test atletici decisivi. Pochi allenamenti: rischio gestione ma il titolare è lui.</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="F16" s="35" t="inlineStr">
         <is>
-          <t>In uscita (Marsiglia)</t>
+          <t>Fuori progetto (resta)</t>
         </is>
       </c>
       <c r="G16" s="35" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="J16" s="36" t="inlineStr">
         <is>
-          <t>PORTA JUVE NEL CAOS: Suzuki saltato (PSG frena), si punta Vicario; Di Gregorio verso il Marsiglia (prestito+obbligo ~15M). Alla 1ª possibile Perin. Porta da NON toccare.</t>
+          <t>NON è partito (Marsiglia non tratta, Monza ci pensa) ma è fuori dal progetto e NON gioca l'esordio: alla 1ª tocca a Perin. Porta Juve nel caos (obiettivo Dibu Martinez). Lasciare.</t>
         </is>
       </c>
     </row>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="F21" s="39" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Titolare (RESTA al Lecce)</t>
         </is>
       </c>
       <c r="G21" s="39" t="inlineStr">
@@ -4778,7 +4778,7 @@
       </c>
       <c r="J21" s="41" t="inlineStr">
         <is>
-          <t>MV 6,4, il '6 politico' — MA è il vice-Meret designato dal NAPOLI: verificare che resti titolare del Lecce prima di pagarlo.</t>
+          <t>RIBALTONE: ha rifiutato il ruolo di vice al Napoli e alla Roma — resta capitano e titolare del Lecce (parte Fruchtl). Torna pienamente comprabile: MV 6,4.</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="F23" s="39" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G23" s="39" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="J23" s="41" t="inlineStr">
         <is>
-          <t>Spalla ko MA in gruppo dal 13/8, obiettivo 1ª (salta solo la Coppa). Selvik non arriva. Low cost n.1 del reparto: verificare i convocati il 21/8.</t>
+          <t>RECUPERATO: titolare in Coppa col Padova (15/8), spalla ok. Low cost n.1 del reparto confermato.</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="F24" s="35" t="inlineStr">
         <is>
-          <t>Titolare (~80%)</t>
+          <t>Titolare (~75%)</t>
         </is>
       </c>
       <c r="G24" s="35" t="inlineStr">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="J24" s="36" t="inlineStr">
         <is>
-          <t>GERARCHIA RISOLTA: riscattato, titolare di Aquilani, Turati vice, Satalino fuori. Prezzo ancora schiacciato dal caos percepito = occasione.</t>
+          <t>Riscattato; Turati in USCITA (Samp) quindi vice ignoto. CalcioDangolo/SOS tengono il ballottaggio formalmente aperto: prezzo ancora schiacciato = occasione. Test: Cesena 17/8.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="F30" s="35" t="inlineStr">
         <is>
-          <t>Al PSG</t>
+          <t>In uscita (Aston Villa)</t>
         </is>
       </c>
       <c r="G30" s="35" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="J30" s="36" t="inlineStr">
         <is>
-          <t>Ceduto al PSG (~35M, non convocato in Coppa) e il prestito alla Juve È SALTATO: via dall'Italia. Depennare.</t>
+          <t>PSG SALTATO il 15/8 (commissioni): ora Aston Villa, che Suzuki preferisce. In ogni caso via dall'Italia: depennare.</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="J34" s="36" t="inlineStr">
         <is>
-          <t>Pista araba sfumata: ora Hull City/Besiktas (ADL chiede 15-18M). Solo da 3° a 1.</t>
+          <t>Proposto alla JUVE come contropartita per Gatti (15M); Hull raffreddata. Solo da 3° a 1.</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="J35" s="41" t="inlineStr">
         <is>
-          <t>Può soffiare la titolarità a Palmisani nel Frosinone: chiamata a 1-2 che può fruttare</t>
+          <t>Ballottaggio vero 45/55 con Palmisani ('decisione a ridosso' — Alvini): la chiamata a 1-2 resta sensata in coppia.</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5348,7 @@
       </c>
       <c r="F36" s="35" t="inlineStr">
         <is>
-          <t>Titolare (Suzuki al PSG)</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="J36" s="36" t="inlineStr">
         <is>
-          <t>Titolare col via libera Suzuki-PSG (transizione in corso), Daffara ko. Ormai noto: non arriverà a 1.</t>
+          <t>Titolare in Coppa (2-0 Catania). MA Daffara recuperato (in panchina): possibile alternanza più avanti. Alla 1ª è lui.</t>
         </is>
       </c>
     </row>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="F37" s="39" t="inlineStr">
         <is>
-          <t>Possibile titolare 1ª</t>
+          <t>Titolare 1ª (~70%)</t>
         </is>
       </c>
       <c r="G37" s="39" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="J37" s="41" t="inlineStr">
         <is>
-          <t>Con la porta Juve nel caos è LUI il candidato per la 1ª (alternanza dichiarata da Spalletti, titolare col Palermo): a 1-2 crediti scommessa sensata in attesa di Vicario.</t>
+          <t>Con Suzuki saltato, Vicario raffreddato e Dibu Martinez lontano, alla 1ª col Frosinone gioca LUI. Chiamata da 2-3 crediti con upside reale.</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="F38" s="35" t="inlineStr">
         <is>
-          <t>Favorito (~65%)</t>
+          <t>Favorito (~55%)</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="J38" s="36" t="inlineStr">
         <is>
-          <t>Titolare nelle ultime 2 amichevoli (Desplanches entra al 70'): più avanti di quanto si creda. Scommessa da 1-2.</t>
+          <t>Titolare in Coppa il 16/8 ma il margine è sceso: 55/45 su Desplanches, decisione sempre a ridosso.</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="F41" s="39" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Recuperato (vice)</t>
         </is>
       </c>
       <c r="G41" s="39" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="J41" s="41" t="inlineStr">
         <is>
-          <t>In corsa per la porta del Parma in caso di cessione di Suzuki</t>
+          <t>RECUPERATO: in panchina in Coppa. Vice di Corvi con possibile alternanza futura: da 1 credito ha senso.</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="F43" s="39" t="inlineStr">
         <is>
-          <t>Ballottaggio a 3</t>
+          <t>In uscita (Samp)</t>
         </is>
       </c>
       <c r="G43" s="39" t="inlineStr">
@@ -5670,11 +5670,11 @@
         </is>
       </c>
       <c r="I43" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" s="41" t="inlineStr">
         <is>
-          <t>Porta Toro IRRISOLTA: Perri arrivato ma non listato; fonti spaccate tra Mascardi e Paleari. Evitare in blocco.</t>
+          <t>In Coppa ha giocato MASCARDI (Paleari panchina) e Perri ha firmato: Paleari verso la Sampdoria. NON comprare.</t>
         </is>
       </c>
     </row>
@@ -5827,7 +5827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="J14" s="36" t="inlineStr">
         <is>
-          <t>Stones favorito 60/40 nelle probabili: ballottaggio confermato, paga mezza fascia sotto.</t>
+          <t>Titolare col Betis (15/8): il 60/40 per Stones non è confermato dal campo. Paga mezza fascia sotto ed è vivo.</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
       </c>
       <c r="F24" s="35" t="inlineStr">
         <is>
-          <t>Favorito su Joao Mario</t>
+          <t>Ballottaggio (panchina in Coppa)</t>
         </is>
       </c>
       <c r="G24" s="35" t="inlineStr">
@@ -6670,11 +6670,11 @@
         </is>
       </c>
       <c r="I24" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J24" s="36" t="inlineStr">
         <is>
-          <t>RIBALTONE: nettamente favorito (Joao Mario terzo). Resta rischio mercato (Milan) e 7 gialli/anno: sconto sì, saldo estremo no.</t>
+          <t>CAPOVOLTO DAL CAMPO: Joao Mario titolare in Coppa (assist), Dodò dentro al 46'. Mercato fermo (rinnovo-ponte allo studio). Solo a forte sconto.</t>
         </is>
       </c>
     </row>
@@ -7350,7 +7350,7 @@
       </c>
       <c r="J41" s="41" t="inlineStr">
         <is>
-          <t>Titolare nelle probabili (con Akanji e Bastoni) ma 60/40 su Bisseck: non pagarlo da inamovibile.</t>
+          <t>Col Betis è partito Bisseck titolare (Stones gol da subentrato): ballottaggio vero, non pagarlo da inamovibile.</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="F42" s="35" t="inlineStr">
         <is>
-          <t>In dubbio (muscolare)</t>
+          <t>Recuperato</t>
         </is>
       </c>
       <c r="G42" s="35" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="J42" s="36" t="inlineStr">
         <is>
-          <t>Recuperato e convocato (14/8) ma muscolo incerto, Tomori pronto. E 9 gialli nel 24/25: fairplay mediocre.</t>
+          <t>A disposizione ed entrato col Man United (15/8). Resta il malus 9 gialli nel 24/25.</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="F54" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Fuori dall'XI atteso</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
@@ -7846,11 +7846,11 @@
         </is>
       </c>
       <c r="I54" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J54" s="36" t="inlineStr">
         <is>
-          <t>Sky low cost: MV ~6,5 con zero hype e solo 3 gialli in 34 gare — titolarità + fairplay a prezzo minimo.</t>
+          <t>DECLASSATO: il Como ha preso Chalobah e l'XI atteso dà Chalobah-Ramon centrali. Solo a 1-2 da copertura.</t>
         </is>
       </c>
     </row>
@@ -7876,7 +7876,7 @@
       </c>
       <c r="F55" s="39" t="inlineStr">
         <is>
-          <t>Titolare Atalanta</t>
+          <t>Titolare Atalanta (listato)</t>
         </is>
       </c>
       <c r="G55" s="39" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="J55" s="41" t="inlineStr">
         <is>
-          <t>UFFICIALE all'Atalanta (13/8, 22M+3) e TITOLARE nel terzetto delle probabili: occasione di listone, listato ancora Udinese.</t>
+          <t>Ora listato ATALANTA (Qt 7, FVM 20): titolare nel terzetto atteso di Sarri. Occasione confermata.</t>
         </is>
       </c>
     </row>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="F56" s="35" t="inlineStr">
         <is>
-          <t>Verso la Juve</t>
+          <t>Juve (visite 16/8)</t>
         </is>
       </c>
       <c r="G56" s="35" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="J56" s="36" t="inlineStr">
         <is>
-          <t>In chiusura con la Juve (~20M, visite 15-16/8): se ufficiale è in ballottaggio con Kelly da titolare bianconero. Comprare solo la notizia confermata.</t>
+          <t>Visite il 16/8, 20M+bonus: in ufficializzazione. In ballottaggio con Kelly; il buco che lascia al Bologna apre a Vitik/Heggem.</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="F58" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare (nuovo XI)</t>
         </is>
       </c>
       <c r="G58" s="35" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J58" s="36" t="inlineStr">
         <is>
-          <t>Nuovo acquisto Como, titolare designato</t>
+          <t>Ufficiale dal Chelsea: centrale titolare nell'XI atteso con Ramon. Il vero acquisto-Como del reparto.</t>
         </is>
       </c>
     </row>
@@ -8396,7 +8396,7 @@
       </c>
       <c r="F68" s="35" t="inlineStr">
         <is>
-          <t>Titolare (~70%)</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G68" s="35" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J68" s="36" t="inlineStr">
         <is>
-          <t>Triplo hit (FantaMaster, Sky, SOS): quinto destro con Zanoli ko fino a ottobre, assist e piazzati in rotazione.</t>
+          <t>90' in Coppa col Padova: confermato dal campo. Piazzati in rotazione.</t>
         </is>
       </c>
     </row>
@@ -8484,7 +8484,7 @@
       </c>
       <c r="F70" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Ballottaggio (~50/50)</t>
         </is>
       </c>
       <c r="G70" s="35" t="inlineStr">
@@ -8498,11 +8498,11 @@
         </is>
       </c>
       <c r="I70" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J70" s="36" t="inlineStr">
         <is>
-          <t>Titolare all'avvio (70/30 su Holm ko al soleo), 2 gialli in 32: posto + fairplay.</t>
+          <t>Holm recuperato (37' col Pisa + Brighton) punta la 1ª da titolare: il 70/30 non regge più.</t>
         </is>
       </c>
     </row>
@@ -8616,7 +8616,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Favorito (65%)</t>
+          <t>Ko ginocchio + ipotesi scambio</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -8630,11 +8630,11 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Cauto ottimismo per l'esordio (65/35 su Pedraza) ma è fermo da 3 settimane: condizione da verificare.</t>
+          <t>PEGGIORATO: infiammazione al ginocchio (fuori in Coppa, Pedraza titolare) E ipotesi scambio con Tomori. Solo a saldo estremo.</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="F82" s="35" t="inlineStr">
         <is>
-          <t>Titolare (terzetto)</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G82" s="35" t="inlineStr">
@@ -8978,7 +8978,7 @@
       </c>
       <c r="J82" s="36" t="inlineStr">
         <is>
-          <t>Il nome nuovo più forte del reparto: titolare nella difesa a 3 di Stroppa, classe 2001 ex Southampton.</t>
+          <t>Titolare in Coppa nel terzetto: confermato — ma la difesa del Venezia ha ballato (2 gol in 39').</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="F84" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -9066,7 +9066,7 @@
       </c>
       <c r="J84" s="36" t="inlineStr">
         <is>
-          <t>Titolarità confermata ma BRUCIATO (n.1 low cost FantaMaster, in tutte le liste): alzare il budget.</t>
+          <t>Titolare in Coppa: confermato, ma bruciato — budget su.</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="F89" s="44" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Superato da Hainaut</t>
         </is>
       </c>
       <c r="G89" s="44" t="inlineStr">
@@ -9282,11 +9282,11 @@
         </is>
       </c>
       <c r="I89" s="44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J89" s="44" t="inlineStr">
         <is>
-          <t>Buona chiamata low cost tra le neopromosse</t>
+          <t>DECLASSATO DAL CAMPO: Hainaut titolare in Coppa, Correia dentro al 74'. Solo ultimo slot.</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
       </c>
       <c r="F93" s="39" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G93" s="39" t="inlineStr">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="J93" s="41" t="inlineStr">
         <is>
-          <t>Titolare ma BRUCIATO ('su tutti Bracaglia' — Goal): prezzo in salita. Piazzati di Calò.</t>
+          <t>Titolare in Coppa (16/8) ma bruciato: prezzo in salita.</t>
         </is>
       </c>
     </row>
@@ -9508,23 +9508,23 @@
       </c>
       <c r="B96" s="43" t="inlineStr">
         <is>
-          <t>Obert</t>
+          <t>Halhal</t>
         </is>
       </c>
       <c r="C96" s="35" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D96" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E96" s="10" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F96" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G96" s="35" t="inlineStr">
@@ -9534,15 +9534,15 @@
       </c>
       <c r="H96" s="36" t="inlineStr">
         <is>
-          <t>Punizioni e corner con Fazzini</t>
+          <t>Terzetto Venezia dal campo</t>
         </is>
       </c>
       <c r="I96" s="10" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J96" s="36" t="inlineStr">
         <is>
-          <t>Promosso 'top di squadra' (costerà) MA 9 ammonizioni nel 25/26: piazzati veri, fairplay pessimo.</t>
+          <t>NUOVO DAL CAMPO: terza maglia del terzetto in Coppa (non Moreno). Zero copertura mediatica: sleeper puro.</t>
         </is>
       </c>
     </row>
@@ -9552,23 +9552,23 @@
       </c>
       <c r="B97" s="38" t="inlineStr">
         <is>
-          <t>Kempf</t>
+          <t>Hainaut</t>
         </is>
       </c>
       <c r="C97" s="39" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D97" s="40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E97" s="40" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F97" s="39" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G97" s="39" t="inlineStr">
@@ -9578,15 +9578,15 @@
       </c>
       <c r="H97" s="41" t="inlineStr">
         <is>
-          <t>CS Como</t>
+          <t>Quinto destro Venezia</t>
         </is>
       </c>
       <c r="I97" s="40" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J97" s="41" t="inlineStr">
         <is>
-          <t>Se non preso prima</t>
+          <t>NUOVO DAL CAMPO: quinto destro titolare in Coppa, ballottaggio con Correia risolto a suo favore.</t>
         </is>
       </c>
     </row>
@@ -9596,23 +9596,23 @@
       </c>
       <c r="B98" s="43" t="inlineStr">
         <is>
-          <t>Kaiki</t>
+          <t>Obert</t>
         </is>
       </c>
       <c r="C98" s="35" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D98" s="10" t="n">
         <v>7</v>
       </c>
       <c r="E98" s="10" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F98" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G98" s="35" t="inlineStr">
@@ -9622,15 +9622,15 @@
       </c>
       <c r="H98" s="36" t="inlineStr">
         <is>
-          <t>5 assist nel 2025 da terzino</t>
+          <t>Punizioni e corner con Fazzini</t>
         </is>
       </c>
       <c r="I98" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J98" s="36" t="inlineStr">
         <is>
-          <t>Favorito su Valle (65/35) ma BRUCIATO da 4 fonti: aspettati rilanci.</t>
+          <t>Titolare in Coppa e blindato (rifiutati 10M del Lens). Restano le 9 ammonizioni 25/26: piazzati veri, fairplay pessimo.</t>
         </is>
       </c>
     </row>
@@ -9640,23 +9640,23 @@
       </c>
       <c r="B99" s="38" t="inlineStr">
         <is>
-          <t>Tavares N.</t>
+          <t>Kempf</t>
         </is>
       </c>
       <c r="C99" s="39" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D99" s="40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E99" s="40" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F99" s="39" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G99" s="39" t="inlineStr">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="H99" s="41" t="inlineStr">
         <is>
-          <t>Potenziale assist</t>
+          <t>CS Como</t>
         </is>
       </c>
       <c r="I99" s="40" t="n">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="J99" s="41" t="inlineStr">
         <is>
-          <t>Rischio alto, resa potenziale altissima</t>
+          <t>Se non preso prima</t>
         </is>
       </c>
     </row>
@@ -9684,19 +9684,19 @@
       </c>
       <c r="B100" s="43" t="inlineStr">
         <is>
-          <t>Biraghi</t>
+          <t>Kaiki</t>
         </is>
       </c>
       <c r="C100" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D100" s="10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E100" s="10" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F100" s="35" t="inlineStr">
         <is>
@@ -9710,15 +9710,15 @@
       </c>
       <c r="H100" s="36" t="inlineStr">
         <is>
-          <t>Tutti i piazzati del Torino</t>
+          <t>5 assist nel 2025 da terzino</t>
         </is>
       </c>
       <c r="I100" s="10" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J100" s="36" t="inlineStr">
         <is>
-          <t>Una stagione intera da titolare può riportarlo ad alti livelli</t>
+          <t>Favorito su Valle (65/35) ma BRUCIATO da 4 fonti: aspettati rilanci.</t>
         </is>
       </c>
     </row>
@@ -9728,23 +9728,23 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Celik</t>
+          <t>Tavares N.</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E101" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Ballottaggio</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Potenziale assist</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Se non preso come D5</t>
+          <t>Rischio alto, resa potenziale altissima</t>
         </is>
       </c>
     </row>
@@ -9772,19 +9772,19 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Jimenez A.</t>
+          <t>Biraghi</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E102" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -9798,15 +9798,15 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Tutti i piazzati del Torino</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Se non preso come D6</t>
+          <t>Una stagione intera da titolare può riportarlo ad alti livelli</t>
         </is>
       </c>
     </row>
@@ -9816,19 +9816,19 @@
       </c>
       <c r="B103" s="44" t="inlineStr">
         <is>
-          <t>Norton-Cuffy</t>
+          <t>Celik</t>
         </is>
       </c>
       <c r="C103" s="44" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D103" s="44" t="n">
         <v>8</v>
       </c>
       <c r="E103" s="44" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F103" s="44" t="inlineStr">
         <is>
@@ -9842,11 +9842,11 @@
       </c>
       <c r="H103" s="44" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="I103" s="44" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J103" s="44" t="inlineStr">
         <is>
@@ -9860,23 +9860,23 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Monterisi</t>
+          <t>Jimenez A.</t>
         </is>
       </c>
       <c r="C104" s="35" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D104" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E104" s="10" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F104" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G104" s="35" t="inlineStr">
@@ -9886,15 +9886,15 @@
       </c>
       <c r="H104" s="36" t="inlineStr">
         <is>
-          <t>5 assist in B, sale sui piazzati</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="I104" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J104" s="36" t="inlineStr">
         <is>
-          <t>Capitano e perno centrale del Frosinone promosso.</t>
+          <t>Se non preso come D6</t>
         </is>
       </c>
     </row>
@@ -9904,23 +9904,23 @@
       </c>
       <c r="B105" s="38" t="inlineStr">
         <is>
-          <t>Calvani</t>
+          <t>Norton-Cuffy</t>
         </is>
       </c>
       <c r="C105" s="39" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D105" s="40" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E105" s="40" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F105" s="39" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G105" s="39" t="inlineStr">
@@ -9930,15 +9930,15 @@
       </c>
       <c r="H105" s="41" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="I105" s="40" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J105" s="41" t="inlineStr">
         <is>
-          <t>Scommessa pura tra le neopromosse</t>
+          <t>Se non preso come D5</t>
         </is>
       </c>
     </row>
@@ -9948,235 +9948,235 @@
       </c>
       <c r="B106" s="43" t="inlineStr">
         <is>
+          <t>Monterisi</t>
+        </is>
+      </c>
+      <c r="C106" s="35" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E106" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="F106" s="35" t="inlineStr">
+        <is>
+          <t>Titolare (campo)</t>
+        </is>
+      </c>
+      <c r="G106" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H106" s="36" t="inlineStr">
+        <is>
+          <t>5 assist in B, sale sui piazzati</t>
+        </is>
+      </c>
+      <c r="I106" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J106" s="36" t="inlineStr">
+        <is>
+          <t>Titolare in Coppa (16/8): capitano e perno, sale sui piazzati.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>15</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Calvani</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>4</v>
+      </c>
+      <c r="E107" t="n">
+        <v>10</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>2</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Scommessa pura tra le neopromosse</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>16</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
           <t>Perez M.</t>
         </is>
       </c>
-      <c r="C106" s="35" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>Lecce</t>
         </is>
       </c>
-      <c r="D106" s="10" t="n">
+      <c r="D108" t="n">
         <v>1</v>
       </c>
-      <c r="E106" s="10" t="n">
+      <c r="E108" t="n">
         <v>1</v>
       </c>
-      <c r="F106" s="35" t="inlineStr">
+      <c r="F108" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="G106" s="35" t="inlineStr">
+      <c r="G108" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H106" s="36" t="inlineStr">
+      <c r="H108" t="inlineStr">
         <is>
           <t>Lecce</t>
         </is>
       </c>
-      <c r="I106" s="10" t="n">
+      <c r="I108" t="n">
         <v>1</v>
       </c>
-      <c r="J106" s="36" t="inlineStr">
+      <c r="J108" t="inlineStr">
         <is>
           <t>Tappabuchi a 1</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="37" t="n"/>
-      <c r="B107" s="38" t="n"/>
-      <c r="C107" s="39" t="n"/>
-      <c r="D107" s="40" t="n"/>
-      <c r="E107" s="40" t="n"/>
-      <c r="F107" s="39" t="n"/>
-      <c r="G107" s="39" t="n"/>
-      <c r="H107" s="41" t="n"/>
-      <c r="I107" s="40" t="n"/>
-      <c r="J107" s="41" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="55" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="37" t="n"/>
+      <c r="B109" s="38" t="n"/>
+      <c r="C109" s="39" t="n"/>
+      <c r="D109" s="40" t="n"/>
+      <c r="E109" s="40" t="n"/>
+      <c r="F109" s="39" t="n"/>
+      <c r="G109" s="39" t="n"/>
+      <c r="H109" s="41" t="n"/>
+      <c r="I109" s="40" t="n"/>
+      <c r="J109" s="41" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="55" t="inlineStr">
         <is>
           <t>SLOT D8 — Scommessa / parcheggio infortunati · budget consigliato: 3</t>
         </is>
       </c>
-      <c r="B108" s="56" t="n"/>
-      <c r="C108" s="56" t="n"/>
-      <c r="D108" s="56" t="n"/>
-      <c r="E108" s="56" t="n"/>
-      <c r="F108" s="56" t="n"/>
-      <c r="G108" s="56" t="n"/>
-      <c r="H108" s="56" t="n"/>
-      <c r="I108" s="56" t="n"/>
-      <c r="J108" s="57" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="12" t="inlineStr">
+      <c r="B110" s="56" t="n"/>
+      <c r="C110" s="56" t="n"/>
+      <c r="D110" s="56" t="n"/>
+      <c r="E110" s="56" t="n"/>
+      <c r="F110" s="56" t="n"/>
+      <c r="G110" s="56" t="n"/>
+      <c r="H110" s="56" t="n"/>
+      <c r="I110" s="56" t="n"/>
+      <c r="J110" s="57" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="12" t="inlineStr">
         <is>
           <t>Priorità</t>
         </is>
       </c>
-      <c r="B109" s="58" t="inlineStr">
+      <c r="B111" s="58" t="inlineStr">
         <is>
           <t>Giocatore</t>
         </is>
       </c>
-      <c r="C109" s="12" t="inlineStr">
+      <c r="C111" s="12" t="inlineStr">
         <is>
           <t>Squadra</t>
         </is>
       </c>
-      <c r="D109" s="59" t="inlineStr">
+      <c r="D111" s="59" t="inlineStr">
         <is>
           <t>Qt.A</t>
         </is>
       </c>
-      <c r="E109" s="59" t="inlineStr">
+      <c r="E111" s="59" t="inlineStr">
         <is>
           <t>FVM</t>
         </is>
       </c>
-      <c r="F109" s="12" t="inlineStr">
+      <c r="F111" s="12" t="inlineStr">
         <is>
           <t>Titolarità</t>
         </is>
       </c>
-      <c r="G109" s="12" t="inlineStr">
+      <c r="G111" s="12" t="inlineStr">
         <is>
           <t>Rigorista</t>
         </is>
       </c>
-      <c r="H109" s="60" t="inlineStr">
+      <c r="H111" s="60" t="inlineStr">
         <is>
           <t>Bonus attesi / punti di forza</t>
         </is>
       </c>
-      <c r="I109" s="59" t="inlineStr">
+      <c r="I111" s="59" t="inlineStr">
         <is>
           <t>Prezzo max</t>
         </is>
       </c>
-      <c r="J109" s="60" t="inlineStr">
+      <c r="J111" s="60" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="B110" s="43" t="inlineStr">
-        <is>
-          <t>Hien</t>
-        </is>
-      </c>
-      <c r="C110" s="35" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="D110" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E110" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="F110" s="35" t="inlineStr">
-        <is>
-          <t>Rientro ottobre</t>
-        </is>
-      </c>
-      <c r="G110" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H110" s="36" t="inlineStr">
-        <is>
-          <t>Top a regime</t>
-        </is>
-      </c>
-      <c r="I110" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J110" s="36" t="inlineStr">
-        <is>
-          <t>Rientro spostato a ottobre (~6ª) e 10 gialli nel 24/25: solo parcheggio a 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="37" t="n">
-        <v>2</v>
-      </c>
-      <c r="B111" s="38" t="inlineStr">
-        <is>
-          <t>Buongiorno</t>
-        </is>
-      </c>
-      <c r="C111" s="39" t="inlineStr">
-        <is>
-          <t>Napoli</t>
-        </is>
-      </c>
-      <c r="D111" s="40" t="n">
-        <v>7</v>
-      </c>
-      <c r="E111" s="40" t="n">
-        <v>18</v>
-      </c>
-      <c r="F111" s="39" t="inlineStr">
-        <is>
-          <t>Rientro dic-gen?</t>
-        </is>
-      </c>
-      <c r="G111" s="39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H111" s="41" t="inlineStr">
-        <is>
-          <t>Top a regime</t>
-        </is>
-      </c>
-      <c r="I111" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="J111" s="41" t="inlineStr">
-        <is>
-          <t>Fonti tra ottobre e dicembre-gennaio: prudenzialmente mezzo girone. Solo a 1.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B112" s="43" t="inlineStr">
         <is>
-          <t>Biraghi</t>
+          <t>Hien</t>
         </is>
       </c>
       <c r="C112" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D112" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E112" s="10" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F112" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Rientro ottobre</t>
         </is>
       </c>
       <c r="G112" s="35" t="inlineStr">
@@ -10186,41 +10186,41 @@
       </c>
       <c r="H112" s="36" t="inlineStr">
         <is>
-          <t>Piazzati</t>
+          <t>Top a regime</t>
         </is>
       </c>
       <c r="I112" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J112" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come D7</t>
+          <t>Rientro spostato a ottobre (~6ª) e 10 gialli nel 24/25: solo parcheggio a 1.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B113" s="38" t="inlineStr">
         <is>
-          <t>Bracaglia</t>
+          <t>Buongiorno</t>
         </is>
       </c>
       <c r="C113" s="39" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D113" s="40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E113" s="40" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F113" s="39" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Rientro dic-gen?</t>
         </is>
       </c>
       <c r="G113" s="39" t="inlineStr">
@@ -10230,38 +10230,38 @@
       </c>
       <c r="H113" s="41" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Top a regime</t>
         </is>
       </c>
       <c r="I113" s="40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J113" s="41" t="inlineStr">
         <is>
-          <t>Se non preso prima</t>
+          <t>Fonti tra ottobre e dicembre-gennaio: prudenzialmente mezzo girone. Solo a 1.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="B114" s="43" t="inlineStr">
+        <is>
+          <t>Biraghi</t>
+        </is>
+      </c>
+      <c r="C114" s="35" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E114" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B114" s="43" t="inlineStr">
-        <is>
-          <t>Correia T.</t>
-        </is>
-      </c>
-      <c r="C114" s="35" t="inlineStr">
-        <is>
-          <t>Venezia</t>
-        </is>
-      </c>
-      <c r="D114" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E114" s="10" t="n">
-        <v>12</v>
-      </c>
       <c r="F114" s="35" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -10274,7 +10274,7 @@
       </c>
       <c r="H114" s="36" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Piazzati</t>
         </is>
       </c>
       <c r="I114" s="10" t="n">
@@ -10282,121 +10282,121 @@
       </c>
       <c r="J114" s="36" t="inlineStr">
         <is>
+          <t>Se non preso come D7</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B115" s="38" t="inlineStr">
+        <is>
+          <t>Bracaglia</t>
+        </is>
+      </c>
+      <c r="C115" s="39" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="D115" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E115" s="40" t="n">
+        <v>11</v>
+      </c>
+      <c r="F115" s="39" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G115" s="39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H115" s="41" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="I115" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="J115" s="41" t="inlineStr">
+        <is>
           <t>Se non preso prima</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>6</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Marin R.</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Napoli</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>2</v>
-      </c>
-      <c r="E115" t="n">
-        <v>6</v>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Titolare per emergenza</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="B116" s="43" t="inlineStr">
+        <is>
+          <t>Correia T.</t>
+        </is>
+      </c>
+      <c r="C116" s="35" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E116" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F116" s="35" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G116" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>Titolare del Napoli fino a ottobre</t>
-        </is>
-      </c>
-      <c r="I115" t="n">
-        <v>3</v>
-      </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>Buongiorno+Beukema+Marianucci out: titolare confermato dalle probabili. A Qt 2. Occhio all'arrivo di Badiashile.</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>7</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Calvani</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
+      <c r="H116" s="36" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="I116" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E116" t="n">
-        <v>10</v>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="I116" t="n">
-        <v>2</v>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>Scommessa a 1-2</t>
+      <c r="J116" s="36" t="inlineStr">
+        <is>
+          <t>Se non preso prima</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Perez M.</t>
+          <t>Marin R.</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E117" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Titolare per emergenza</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -10406,41 +10406,41 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Titolare del Napoli fino a ottobre</t>
         </is>
       </c>
       <c r="I117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Tappabuchi</t>
+          <t>Titolare confermato in coppia con Rrahmani. Unico rischio: Badiashile (visite martedì 18/8, non ancora listato).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tavares N.</t>
+          <t>Calvani</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E118" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10450,41 +10450,41 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Assist</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="I118" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Scommessa di lusso</t>
+          <t>Scommessa a 1-2</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Mangas</t>
+          <t>Perez M.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E119" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10494,41 +10494,41 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="I119" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Se non preso prima</t>
+          <t>Tappabuchi</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Mitaj</t>
+          <t>Tavares N.</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E120" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Ballottaggio</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -10538,37 +10538,37 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Quinto sinistro nuovo di De Rossi</t>
+          <t>Assist</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Favorito ~55% su Ellertsson ma BRUCIATO (FantaMaster, Goal, Sisal): non più a 1-2.</t>
+          <t>Scommessa di lusso</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Marusic</t>
+          <t>Mangas</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D121" t="n">
         <v>6</v>
       </c>
       <c r="E121" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -10582,57 +10582,145 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Usato sicuro sulle fasce</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="I121" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Scommessa citata dalle guide: esperienza e titolarità nella Lazio</t>
+          <t>Se non preso prima</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
+        <v>11</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Mitaj</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>4</v>
+      </c>
+      <c r="E122" t="n">
+        <v>9</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Incerto</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Quinto sinistro nuovo di De Rossi</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>3</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Probabili di Coppa discordanti (una lo esclude dal terzetto): verificare l'XI vero di Genoa-Ascoli prima di pagarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>12</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Marusic</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>6</v>
+      </c>
+      <c r="E123" t="n">
+        <v>20</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Usato sicuro sulle fasce</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>5</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Scommessa citata dalle guide: esperienza e titolarità nella Lazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
         <v>13</v>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B124" t="inlineStr">
         <is>
           <t>Kempf</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>Como</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D124" t="n">
         <v>5</v>
       </c>
-      <c r="E122" t="n">
+      <c r="E124" t="n">
         <v>13</v>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="F124" t="inlineStr">
         <is>
           <t>Altissima</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr">
+      <c r="G124" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr">
+      <c r="H124" t="inlineStr">
         <is>
           <t>Como</t>
         </is>
       </c>
-      <c r="I122" t="n">
+      <c r="I124" t="n">
         <v>7</v>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="J124" t="inlineStr">
         <is>
           <t>Se non preso prima</t>
         </is>
@@ -10644,10 +10732,10 @@
     <mergeCell ref="A46:J46"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A62:J62"/>
+    <mergeCell ref="A76:J76"/>
     <mergeCell ref="A91:J91"/>
+    <mergeCell ref="A110:J110"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A76:J76"/>
-    <mergeCell ref="A108:J108"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -10660,7 +10748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10945,7 +11033,7 @@
       </c>
       <c r="F10" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Rientro tardivo</t>
         </is>
       </c>
       <c r="G10" s="35" t="inlineStr">
@@ -10959,11 +11047,11 @@
         </is>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J10" s="36" t="inlineStr">
         <is>
-          <t>Perno del Milan di Amorim</t>
+          <t>Rientrato a Milanello solo il 16/8 (post-Mondiale): Jashari gli è passato davanti per l'avvio. Scontare le prime giornate.</t>
         </is>
       </c>
     </row>
@@ -11450,7 +11538,7 @@
       </c>
       <c r="G23" s="39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì (1° unanime)</t>
         </is>
       </c>
       <c r="H23" s="41" t="inlineStr">
@@ -11463,7 +11551,7 @@
       </c>
       <c r="J23" s="41" t="inlineStr">
         <is>
-          <t>Capitano ma rigori NON garantiti (Sky dà Cataldi) e fairplay pessimo: 6 gialli + 1 rosso nel 25/26, 10 nel 24/25.</t>
+          <t>CORRETTO: rigorista 1° UNANIME (6/6 fonti, anche Sky — la lettura 'Cataldi 1°' era errata). Resta il fairplay pessimo e l'insidia Pinamonti se arriva. Prezzo destinato a salire.</t>
         </is>
       </c>
     </row>
@@ -11875,7 +11963,7 @@
       </c>
       <c r="J34" s="36" t="inlineStr">
         <is>
-          <t>Pacchetto bonus completo + fairplay pulito, ma il minutaggio con Allegri non è garantito (Anguissa insidia).</t>
+          <t>Rigorista 1° per 4 fonti (SOS/Goal ferme a Lukaku: ignorare) ma il minutaggio con Allegri resta APERTO (segnali contrastanti su KDB vs Anguissa). Semi-top.</t>
         </is>
       </c>
     </row>
@@ -11906,7 +11994,7 @@
       </c>
       <c r="G35" s="39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì (1° unanime)</t>
         </is>
       </c>
       <c r="H35" s="41" t="inlineStr">
@@ -11919,7 +12007,7 @@
       </c>
       <c r="J35" s="41" t="inlineStr">
         <is>
-          <t>Gerarchia rigori apertissima e 7 cartellini nel 25/26: doppio sconto d'obbligo.</t>
+          <t>Rigorista 1° unanime; malus disciplina confermato (6 gialli + 1 rosso nel 25/26). Sconto solo per il fairplay, non più per i rigori.</t>
         </is>
       </c>
     </row>
@@ -12051,7 +12139,7 @@
       </c>
       <c r="J38" s="36" t="inlineStr">
         <is>
-          <t>RESTA (zero offerte formali) ed è 'certo del posto' (14/8): rigorista favorito. Mercato aperto fino all'1/9: ultimo check il giorno dell'asta.</t>
+          <t>In gol al 2' in Coppa, rigorista confermato. Di fatto sul mercato (15-20M, sondaggio Atalanta) ma zero offerte depositate: comprare con un occhio all'1/9.</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12271,7 @@
       </c>
       <c r="J41" s="41" t="inlineStr">
         <is>
-          <t>RIDIMENSIONATO: fuori in Coppa Italia ('formazione collaudata'), Atta favorito. 3/3 sui rigori al River: prospetto, non titolare subito.</t>
+          <t>Subentro al 58' anche in Coppa: confermato ridimensionato, Atta davanti. Metà prezzo.</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12903,7 @@
       </c>
       <c r="J57" s="41" t="inlineStr">
         <is>
-          <t>LA scommessa del Genoa (FantaMaster) e n.1 PazziDiFanta: 1° sulle punizioni, titolare ~65% — BRUCIATO, budget su.</t>
+          <t>Titolare nella probabile di Coppa, 1° sulle punizioni: confermato ma bruciato.</t>
         </is>
       </c>
     </row>
@@ -13095,7 +13183,7 @@
       </c>
       <c r="J65" s="41" t="inlineStr">
         <is>
-          <t>Cambio ruolo A→C il più vantaggioso del listone MA Rowe nettamente favorito (80/20): bonus da subentri.</t>
+          <t>RIVALUTATO: titolare col Brighton (Rowe dentro al 62'): l'80/20 per Rowe non è più netto. Cambio ruolo A→C sempre d'oro.</t>
         </is>
       </c>
     </row>
@@ -13297,7 +13385,7 @@
       </c>
       <c r="F70" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G70" s="35" t="inlineStr">
@@ -13315,7 +13403,7 @@
       </c>
       <c r="J70" s="36" t="inlineStr">
         <is>
-          <t>Perno del Torino di Baroni</t>
+          <t>90' da sotto-punta in Coppa con Vlasic, mai sostituito: perno di ABATE (non Baroni). Il low cost C del Toro è lui.</t>
         </is>
       </c>
     </row>
@@ -13551,7 +13639,7 @@
       </c>
       <c r="J77" s="41" t="inlineStr">
         <is>
-          <t>Più minutaggio con l'addio di Atta, accanto a Zaniolo; 1 giallo in 31: pulito.</t>
+          <t>Titolare in Coppa accanto a Zaniolo: confermato dal campo.</t>
         </is>
       </c>
     </row>
@@ -13577,7 +13665,7 @@
       </c>
       <c r="F78" s="35" t="inlineStr">
         <is>
-          <t>In dubbio (schiena)</t>
+          <t>Recuperato</t>
         </is>
       </c>
       <c r="G78" s="35" t="inlineStr">
@@ -13595,7 +13683,7 @@
       </c>
       <c r="J78" s="36" t="inlineStr">
         <is>
-          <t>In dubbio per la 1ª E recidivo dei cartellini (7 gialli nel 25/26 e nel 24/25): doppio malus.</t>
+          <t>MIGLIORATO: la schiena è sciatalgia in risoluzione, esordio con la Roma non a rischio. Resta il malus cartellini (7 gialli x2 stagioni).</t>
         </is>
       </c>
     </row>
@@ -13635,11 +13723,11 @@
         </is>
       </c>
       <c r="I79" s="40" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J79" s="41" t="inlineStr">
         <is>
-          <t>Triplo hit consigli (FantaMaster, PazziDiFanta, Goal): titolare nella mediana di Grosso.</t>
+          <t>PROMOSSO: titolare E GOL in Coppa nella mediana di Grosso. Costerà più del previsto.</t>
         </is>
       </c>
     </row>
@@ -14051,7 +14139,7 @@
       </c>
       <c r="J90" s="36" t="inlineStr">
         <is>
-          <t>Tiratore unico del Frosinone (4-3-3 confermato) e rigorista. Sky avverte: 'bonus ridotti in A' — resta il low cost d'oro, senza esagerare.</t>
+          <t>Titolare in Coppa (16/8) nel 4-3-3 confermato: rigori e tutti i piazzati suoi. 5 fonti su 6 lo confermano rigorista.</t>
         </is>
       </c>
     </row>
@@ -14121,7 +14209,7 @@
       </c>
       <c r="F92" s="35" t="inlineStr">
         <is>
-          <t>Firma Lazio il 15/8</t>
+          <t>UFFICIALE Lazio (15/8)</t>
         </is>
       </c>
       <c r="G92" s="35" t="inlineStr">
@@ -14139,7 +14227,7 @@
       </c>
       <c r="J92" s="36" t="inlineStr">
         <is>
-          <t>Sbloccato il 14/8 (prestito 5M + diritto 10M) dopo lo stop della Lega: visite sabato. Mezzala di Gattuso, ballottaggio iniziale con Dele-Bashiru: comprare la notizia senza strapagare.</t>
+          <t>Ufficiale e ora listato Lazio (Qt 7, FVM 55): in Coppa è partito Dele-Bashiru ma Gattuso lo indica titolare col Bologna. Investimento, non low cost.</t>
         </is>
       </c>
     </row>
@@ -14214,7 +14302,7 @@
       </c>
       <c r="G94" s="35" t="inlineStr">
         <is>
-          <t>Alternativa</t>
+          <t>Candidato 1°</t>
         </is>
       </c>
       <c r="H94" s="36" t="inlineStr">
@@ -14227,7 +14315,7 @@
       </c>
       <c r="J94" s="36" t="inlineStr">
         <is>
-          <t>Nel Parma può ereditare i rigori se parte Pellegrino</t>
+          <t>Regista titolare in Coppa e candidato n.1 ai rigori del Parma (F-online) — ma valuta la cessione: comprarlo per i piazzati, monitorare il mercato.</t>
         </is>
       </c>
     </row>
@@ -14253,7 +14341,7 @@
       </c>
       <c r="F95" s="39" t="inlineStr">
         <is>
-          <t>Ballottaggio Sohm</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G95" s="39" t="inlineStr">
@@ -14267,11 +14355,11 @@
         </is>
       </c>
       <c r="I95" s="40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J95" s="41" t="inlineStr">
         <is>
-          <t>Sky lo promuove: specialista di angoli e punizioni (3 gol + 7 assist in B). A 1-2 è un furto se parte titolare.</t>
+          <t>Titolare in Coppa (con Busio e Sohm): specialista piazzati confermato dal campo.</t>
         </is>
       </c>
     </row>
@@ -14341,7 +14429,7 @@
       </c>
       <c r="F97" s="39" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>CONGELATO</t>
         </is>
       </c>
       <c r="G97" s="39" t="inlineStr">
@@ -14355,11 +14443,11 @@
         </is>
       </c>
       <c r="I97" s="40" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J97" s="41" t="inlineStr">
         <is>
-          <t>Titolare nel Venezia, tiro da fuori</t>
+          <t>Né in campo né in panchina in Coppa senza spiegazione (possibile mercato): congelare finché non si chiarisce.</t>
         </is>
       </c>
     </row>
@@ -14403,7 +14491,7 @@
       </c>
       <c r="J98" s="36" t="inlineStr">
         <is>
-          <t>Titolare confermato ovunque ('libertà di svariare'): piazzati sì, rigori verso Kevin Carlos/Maldini.</t>
+          <t>Titolare in Coppa, piazzati confermati — ma i rigori del Cagliari sono di DEIOLA (dal campo).</t>
         </is>
       </c>
     </row>
@@ -14535,7 +14623,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Lussazione della rotula, operato: 2-3 mesi. DEPENNARE. I rigori del Monza passano a Cutrone.</t>
+          <t>Operato, rientro NOVEMBRE. Ancora schierato titolare da 3 aggregatori: non farsi ingannare. DEPENNARE.</t>
         </is>
       </c>
     </row>
@@ -14757,41 +14845,41 @@
       </c>
       <c r="B108" s="43" t="inlineStr">
         <is>
-          <t>Moro N.</t>
+          <t>Deiola</t>
         </is>
       </c>
       <c r="C108" s="35" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D108" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E108" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F108" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare/capitano</t>
         </is>
       </c>
       <c r="G108" s="35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì (dal campo)</t>
         </is>
       </c>
       <c r="H108" s="36" t="inlineStr">
         <is>
-          <t>Spazio nel Bologna</t>
+          <t>RIGORISTA del Cagliari (segnato in Coppa)</t>
         </is>
       </c>
       <c r="I108" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J108" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C6</t>
+          <t>IL COLPO DEL TURNO: unico rigore dei 32esimi calciato e SEGNATO da lui (ribattuto anche dopo annullamento VAR), con Winks e Fazzini in campo. Nessuna guida lo dà. A 2-4 è il furto-rigori dell'asta.</t>
         </is>
       </c>
     </row>
@@ -14801,19 +14889,19 @@
       </c>
       <c r="B109" s="38" t="inlineStr">
         <is>
-          <t>Traorè Hj.</t>
+          <t>Moro N.</t>
         </is>
       </c>
       <c r="C109" s="39" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D109" s="40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E109" s="40" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F109" s="39" t="inlineStr">
         <is>
@@ -14827,7 +14915,7 @@
       </c>
       <c r="H109" s="41" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Spazio nel Bologna</t>
         </is>
       </c>
       <c r="I109" s="40" t="n">
@@ -14835,7 +14923,7 @@
       </c>
       <c r="J109" s="41" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>Se non preso come C6</t>
         </is>
       </c>
     </row>
@@ -14845,23 +14933,23 @@
       </c>
       <c r="B110" s="43" t="inlineStr">
         <is>
-          <t>Schmid</t>
+          <t>Traorè Hj.</t>
         </is>
       </c>
       <c r="C110" s="35" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D110" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E110" s="10" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F110" s="35" t="inlineStr">
         <is>
-          <t>Favorito nel tridente</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G110" s="35" t="inlineStr">
@@ -14871,15 +14959,15 @@
       </c>
       <c r="H110" s="36" t="inlineStr">
         <is>
-          <t>4 gol + 8 assist in Germania</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="I110" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J110" s="36" t="inlineStr">
         <is>
-          <t>FAVORITO (~40%) su Kvernadze e Zerbin per il 3° slot del 4-3-3: quasi nessuno lo conosce. Titolare per fantacalcio.it e PazziDiFanta.</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -14889,7 +14977,7 @@
       </c>
       <c r="B111" s="38" t="inlineStr">
         <is>
-          <t>Calò</t>
+          <t>Schmid</t>
         </is>
       </c>
       <c r="C111" s="39" t="inlineStr">
@@ -14898,14 +14986,14 @@
         </is>
       </c>
       <c r="D111" s="40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E111" s="40" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F111" s="39" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Fuori dall'XI di Coppa</t>
         </is>
       </c>
       <c r="G111" s="39" t="inlineStr">
@@ -14915,15 +15003,15 @@
       </c>
       <c r="H111" s="41" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>4 gol + 8 assist in Germania</t>
         </is>
       </c>
       <c r="I111" s="40" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J111" s="41" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>BOCCIATO DAL CAMPO: non impiegato in Coppa (Fini al suo posto) nonostante gli aggregatori lo diano favorito: sopravvalutato.</t>
         </is>
       </c>
     </row>
@@ -14933,23 +15021,23 @@
       </c>
       <c r="B112" s="43" t="inlineStr">
         <is>
-          <t>Perez K.</t>
+          <t>Fini</t>
         </is>
       </c>
       <c r="C112" s="35" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D112" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E112" s="10" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F112" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare in Coppa</t>
         </is>
       </c>
       <c r="G112" s="35" t="inlineStr">
@@ -14959,7 +15047,7 @@
       </c>
       <c r="H112" s="36" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Tridente Frosinone dal campo</t>
         </is>
       </c>
       <c r="I112" s="10" t="n">
@@ -14967,7 +15055,7 @@
       </c>
       <c r="J112" s="36" t="inlineStr">
         <is>
-          <t>Piazzati del Venezia in canna: da ultimo slot è oro (ballottaggio con Sohm).</t>
+          <t>NUOVO DAL CAMPO: titolare nel tridente di Coppa (16/8) al posto di Schmid/Zerbin. Nessuno lo ha in lista.</t>
         </is>
       </c>
     </row>
@@ -14977,23 +15065,23 @@
       </c>
       <c r="B113" s="38" t="inlineStr">
         <is>
-          <t>Adzic</t>
+          <t>Calò</t>
         </is>
       </c>
       <c r="C113" s="39" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D113" s="40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E113" s="40" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F113" s="39" t="inlineStr">
         <is>
-          <t>Titolare (55/45)</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G113" s="39" t="inlineStr">
@@ -15003,15 +15091,15 @@
       </c>
       <c r="H113" s="41" t="inlineStr">
         <is>
-          <t>2° tiratore di punizioni e corner dietro Berardi</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="I113" s="40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J113" s="41" t="inlineStr">
         <is>
-          <t>Titolare (55/45 su Lipani), gran tiro da fuori — BRUCIATO da 4 fonti: alzare il budget.</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -15021,23 +15109,23 @@
       </c>
       <c r="B114" s="43" t="inlineStr">
         <is>
-          <t>Vergara</t>
+          <t>Perez K.</t>
         </is>
       </c>
       <c r="C114" s="35" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D114" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E114" s="10" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="F114" s="35" t="inlineStr">
         <is>
-          <t>Scommessa (tibia ko)</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G114" s="35" t="inlineStr">
@@ -15047,15 +15135,15 @@
       </c>
       <c r="H114" s="36" t="inlineStr">
         <is>
-          <t>Gol in Champions, corner in rotazione</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="I114" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J114" s="36" t="inlineStr">
         <is>
-          <t>'Una delle scommesse più interessanti' (PlayerManager) a 1-2 crediti — ma contusione alla tibia riacutizzata il 12/8: verificare.</t>
+          <t>Piazzati del Venezia in canna: da ultimo slot è oro (ballottaggio con Sohm).</t>
         </is>
       </c>
     </row>
@@ -15065,23 +15153,23 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Oristanio</t>
+          <t>Adzic</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E115" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>50/50 con Njie</t>
+          <t>Titolare (55/45)</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -15091,15 +15179,15 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2° tiratore piazzati dietro Vlasic</t>
+          <t>2° tiratore di punizioni e corner dietro Berardi</t>
         </is>
       </c>
       <c r="I115" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>50/50 VERO con Njie (il campo dell'8/8 premiava Njie): dualismo da monitorare fino all'asta.</t>
+          <t>APERTO: in Coppa atteso/impiegato Lipani, ma fantacalcio.it dà Adzic titolare alla 1ª: 50/50 vero.</t>
         </is>
       </c>
     </row>
@@ -15109,23 +15197,23 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Milla</t>
+          <t>Vergara</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E116" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Recuperato</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -15135,15 +15223,15 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Gol in Champions, corner in rotazione</t>
         </is>
       </c>
       <c r="I116" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>Rientrato in gruppo: la scommessa a 1-2 torna valida.</t>
         </is>
       </c>
     </row>
@@ -15153,23 +15241,23 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Oristanio</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E117" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Bocciato dal campo</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -15179,15 +15267,15 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>2° tiratore piazzati dietro Vlasic</t>
         </is>
       </c>
       <c r="I117" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Posto fisso + piazzati a 1-2 MA ballottaggio con Sohm (DAZN) e un rosso nel 25/26.</t>
+          <t>Panchina in Coppa, MAI entrato nemmeno a gara chiusa: il posto oggi è di Casadei/Cacciamani. Solo a saldo.</t>
         </is>
       </c>
     </row>
@@ -15197,23 +15285,23 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Aboukhlal</t>
+          <t>Milla</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E118" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Fondo gerarchie</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -15223,15 +15311,15 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Cambio ruolo A→C</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="I118" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>SMENTITO dalle probabili: nessuna fonte lo dà titolare (DAZN lo mette dietro Vlasic/Oristanio/Njie). Solo ultimo slot a 1.</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -15241,7 +15329,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Busio</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -15250,10 +15338,10 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E119" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -15275,7 +15363,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>Posto fisso + piazzati a 1-2 MA ballottaggio con Sohm (DAZN) e un rosso nel 25/26.</t>
         </is>
       </c>
     </row>
@@ -15285,23 +15373,23 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Zhegrova</t>
+          <t>Aboukhlal</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E120" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Fondo gerarchie</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -15311,15 +15399,15 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Cambio ruolo A→C</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Se non preso come C5</t>
+          <t>SMENTITO dalle probabili: nessuna fonte lo dà titolare (DAZN lo mette dietro Vlasic/Oristanio/Njie). Solo ultimo slot a 1.</t>
         </is>
       </c>
     </row>
@@ -15329,23 +15417,23 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Isaksen</t>
+          <t>Busio</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E121" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Alta (post-infortunio)</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -15355,15 +15443,15 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="I121" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Scommessa di lusso se il prezzo crolla</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -15373,39 +15461,127 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>Zhegrova</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>6</v>
+      </c>
+      <c r="E122" t="n">
+        <v>18</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Ballottaggio</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>10</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Se non preso come C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>17</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Isaksen</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>9</v>
+      </c>
+      <c r="E123" t="n">
+        <v>25</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Alta (post-infortunio)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>20</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Scommessa di lusso se il prezzo crolla</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>18</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
           <t>Stankovic A.</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>Inter</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D124" t="n">
         <v>3</v>
       </c>
-      <c r="E122" t="n">
+      <c r="E124" t="n">
         <v>10</v>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="F124" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr">
+      <c r="G124" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr">
+      <c r="H124" t="inlineStr">
         <is>
           <t>Talento Inter</t>
         </is>
       </c>
-      <c r="I122" t="n">
+      <c r="I124" t="n">
         <v>2</v>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="J124" t="inlineStr">
         <is>
           <t>Puro parcheggio a 1: minutaggio da verificare</t>
         </is>
@@ -15433,7 +15609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15604,7 +15780,7 @@
       </c>
       <c r="J7" s="41" t="inlineStr">
         <is>
-          <t>Il 9 FAVORITO (70/30 su Castro, 6/6 probabili) e rigorista di misura. 1 giallo nel 25/26: perfetto anche per il fairplay.</t>
+          <t>CONFERMATO DAL CAMPO: titolare da 9 e rigorista anche col Dortmund (Dybala-Soulé dietro). Il pacchetto regge tutto.</t>
         </is>
       </c>
     </row>
@@ -15648,7 +15824,7 @@
       </c>
       <c r="J8" s="36" t="inlineStr">
         <is>
-          <t>Polpaccio ko: salta l'ultima amichevole, a forte rischio per la 1ª. Top sull'anno, non per l'avvio.</t>
+          <t>Polpaccio: saltato anche il Betis; titolare alla 1ª solo se risolve del tutto. E Lautaro è RECUPERATO: gerarchie d'avvio ribaltate. Top sull'anno, sconto sull'avvio.</t>
         </is>
       </c>
     </row>
@@ -15723,7 +15899,7 @@
       </c>
       <c r="G10" s="35" t="inlineStr">
         <is>
-          <t>1° per le fonti fresche</t>
+          <t>Sì (di fatto alla 1ª)</t>
         </is>
       </c>
       <c r="H10" s="36" t="inlineStr">
@@ -15736,7 +15912,7 @@
       </c>
       <c r="J10" s="36" t="inlineStr">
         <is>
-          <t>Il 9 fisso (unanime) e per FantaMaster/Fantacalcio.it è LUI il rigorista, non Nkunku. Zero dubbi di posto.</t>
+          <t>Titolare e gol col Man United (7,5): con Nkunku FUORI ROSA e Gimenez verso il Porto è il 9 e il rigorista di fatto. Da pagare.</t>
         </is>
       </c>
     </row>
@@ -16456,7 +16632,7 @@
       </c>
       <c r="J28" s="36" t="inlineStr">
         <is>
-          <t>DOPPIO ALLARME 14/8: il Milan apre alla cessione (richiesta giù a 40-45M, Gala pronto) E problema muscolare, in dubbio per la 1ª. Forte sconto o lasciare.</t>
+          <t>Quadricipite (salta lo United) + mercato: il Milan ha ALZATO a 50-60M e rifiuta il prestito con obbligo → permanenza più probabile, ma condizione e ruolo con Amorim tutti da capire. Solo a forte sconto.</t>
         </is>
       </c>
     </row>
@@ -16500,7 +16676,7 @@
       </c>
       <c r="J29" s="41" t="inlineStr">
         <is>
-          <t>Caviglia: preparazione saltata, in dubbio per la 1ª. E un rosso nel 25/26. Scontare.</t>
+          <t>Fonti divise: caviglia che 'si porta dietro da febbraio' e niente gruppo pieno VS Aquilani che assicura 'a disposizione per la 1ª'. Guardare i convocati col Cesena (17/8). Scontare comunque.</t>
         </is>
       </c>
     </row>
@@ -16718,7 +16894,7 @@
       </c>
       <c r="F36" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Ballottaggio 55/45</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -16732,11 +16908,11 @@
         </is>
       </c>
       <c r="I36" s="10" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="J36" s="36" t="inlineStr">
         <is>
-          <t>Titolare designato (70/30 su Piccoli che è VICE, non trequartista) e ZERO cartellini: gol + fairplay.</t>
+          <t>DOPPIO DOWNGRADE: ballottaggio vero con Piccoli (55/45, non 70/30) e prova pessima col Brighton (45', zero tiri, sostituito per l'esordio di Piccoli). Fairplay ok, prezzo da rifare.</t>
         </is>
       </c>
     </row>
@@ -16824,7 +17000,7 @@
       </c>
       <c r="J38" s="36" t="inlineStr">
         <is>
-          <t>Distrazione agli adduttori (12/8): a rischio per la 1ª. Resta il titolare designato a destra: sconto-infortunio.</t>
+          <t>OUT confermato per la 1ª (in dubbio anche 2ª). Due aggregatori lo schierano ancora: comprarlo con lo sconto-infortunio.</t>
         </is>
       </c>
     </row>
@@ -17044,7 +17220,7 @@
       </c>
       <c r="J43" s="41" t="inlineStr">
         <is>
-          <t>Certezza (70/30, Zapata non convocato) e 1 giallo in 32 presenze: voti, gol e fairplay.</t>
+          <t>PROMOSSO DAL CAMPO: gol in Coppa all'8', prima scelta di Abate (Zapata fermo). Voti, gol e fairplay: il segnale più forte del turno.</t>
         </is>
       </c>
     </row>
@@ -17262,7 +17438,7 @@
       </c>
       <c r="F50" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>FUORI ROSA (mercato)</t>
         </is>
       </c>
       <c r="G50" s="35" t="inlineStr">
@@ -17276,11 +17452,11 @@
         </is>
       </c>
       <c r="I50" s="10" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="J50" s="36" t="inlineStr">
         <is>
-          <t>'Unico sicuro del posto' sulla trequarti + 0 cartellini MA rigori contesi con Ramos e ipotesi scambio con Soulè (14/8): semi-top con riserva.</t>
+          <t>Escluso col Man United per scelta tecnica/mercato; scambio con Soulè MORTO ma la Roma lo vuole in prestito (Milan chiede 35M). Rigori di fatto a Ramos. NON comprare finché non si chiarisce.</t>
         </is>
       </c>
     </row>
@@ -17311,7 +17487,7 @@
       </c>
       <c r="G51" s="39" t="inlineStr">
         <is>
-          <t>Sì (3/3)</t>
+          <t>NO (nessun designato)</t>
         </is>
       </c>
       <c r="H51" s="41" t="inlineStr">
@@ -17320,11 +17496,11 @@
         </is>
       </c>
       <c r="I51" s="40" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J51" s="41" t="inlineStr">
         <is>
-          <t>PROMOSSO: Pellegrino ufficiale alla Viola → è il 9 (6/7 probabili) e rigorista del Parma. Comprare prima che il prezzo salga.</t>
+          <t>CORRETTO: titolare + assist in Coppa MA il Parma non ha un rigorista designato (Bernabè candidato) e Lontani (2008, doppietta) insidia i minuti. Pagarlo da titolare, non da rigorista.</t>
         </is>
       </c>
     </row>
@@ -17394,7 +17570,7 @@
       </c>
       <c r="F53" s="39" t="inlineStr">
         <is>
-          <t>Trattativa Lazio rallentata</t>
+          <t>Trattativa Lazio AVANZATA</t>
         </is>
       </c>
       <c r="G53" s="39" t="inlineStr">
@@ -17412,7 +17588,7 @@
       </c>
       <c r="J53" s="41" t="inlineStr">
         <is>
-          <t>Distanza su formula e prezzo (il Sassuolo non scende da 15M): rischio addio reale ma non imminente. Nelle probabili è ancora il 9 del Sassuolo.</t>
+          <t>Sassuolo sceso a 12M, accordo di massima col giocatore, OUT dalla Coppa per mercato. Se va alla Lazio è candidato rigorista biancoceleste (20/24). Non comprarlo da 9 del Sassuolo.</t>
         </is>
       </c>
     </row>
@@ -17482,7 +17658,7 @@
       </c>
       <c r="F55" s="39" t="inlineStr">
         <is>
-          <t>Titolare (65%)</t>
+          <t>Assente in Coppa</t>
         </is>
       </c>
       <c r="G55" s="39" t="inlineStr">
@@ -17496,11 +17672,11 @@
         </is>
       </c>
       <c r="I55" s="40" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J55" s="41" t="inlineStr">
         <is>
-          <t>Fantacalcio.it lo dà 1° RIGORISTA (Maldini 2°), FantaMaster il contrario: gerarchia da verificare all'ultimo. A Qt 13 scommessa-rigori vera.</t>
+          <t>RIDIMENSIONATO: assente in Coppa (non al 100%) e rigori dal campo a Deiola. La scommessa-rigori non esiste più: solo scommessa-posto.</t>
         </is>
       </c>
     </row>
@@ -17544,7 +17720,7 @@
       </c>
       <c r="J56" s="36" t="inlineStr">
         <is>
-          <t>Ipotesi SCAMBIO col Milan (per Nkunku), Gala in agguato, la Roma deve cedere per il FFP: nelle probabili è titolare, ma solo con sconto-mercato.</t>
+          <t>Scambio-Nkunku MORTO e titolare col Dortmund: allarme rientrato a metà (il tema FFP resta, è tra i cedibili con Koné). Sconto-mercato ridotto.</t>
         </is>
       </c>
     </row>
@@ -17584,11 +17760,11 @@
         </is>
       </c>
       <c r="I57" s="40" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J57" s="41" t="inlineStr">
         <is>
-          <t>Coppia con Yeboah CONFERMATA (7/7) e rigori in alternanza — ma BRUCIATO: alzare il budget.</t>
+          <t>DOPPIETTA in Coppa (+ assist di fatto sull'autogol): bruciatissimo, alzare il budget o lasciare. Rigori sempre in alternanza con Rrahmani.</t>
         </is>
       </c>
     </row>
@@ -17632,7 +17808,7 @@
       </c>
       <c r="J58" s="36" t="inlineStr">
         <is>
-          <t>Cambio ruolo C→A svantaggioso MA titolare per fantacalcio.it alla 1ª (Neres out): interessante solo per l'avvio.</t>
+          <t>Titolare atteso a sinistra alla 1ª (Neres out, Lang ko/ai margini): buono per l'avvio nonostante il cambio ruolo C→A svantaggioso.</t>
         </is>
       </c>
     </row>
@@ -17824,7 +18000,7 @@
       </c>
       <c r="J64" s="36" t="inlineStr">
         <is>
-          <t>PROMOSSO: con Pessina operato eredita i RIGORI del Monza, 0 cartellini nel 25/26. Da low cost a semi-gem.</t>
+          <t>Unica punta 90' in Coppa (3-4-2-1: NON coppia con Petagna) e rigorista designato. A secco ma il posto è blindato.</t>
         </is>
       </c>
     </row>
@@ -17912,7 +18088,7 @@
       </c>
       <c r="J66" s="36" t="inlineStr">
         <is>
-          <t>Titolare alla 1ª e 'già in palla', più avanti di Esposito: avvio garantito a Qt 7.</t>
+          <t>Titolare col Betis MA Lautaro recuperato 'scalpita': avvio da co-titolare, non più garantito.</t>
         </is>
       </c>
     </row>
@@ -17943,7 +18119,7 @@
       </c>
       <c r="G67" s="39" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>Conteso (4 fonti lo danno 1°)</t>
         </is>
       </c>
       <c r="H67" s="41" t="inlineStr">
@@ -17952,11 +18128,11 @@
         </is>
       </c>
       <c r="I67" s="40" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J67" s="41" t="inlineStr">
         <is>
-          <t>Dovrebbe prendersi la responsabilità dal dischetto</t>
+          <t>Fuori dalla probabile di Coppa (posto a Geubbels) MA 4 fonti su 7 lo danno 1° rigorista: scommessa contro-intuitiva a 3-5.</t>
         </is>
       </c>
     </row>
@@ -18000,7 +18176,7 @@
       </c>
       <c r="J68" s="36" t="inlineStr">
         <is>
-          <t>Non convocato in Coppa, dietro Simeone e Adams: lasciarlo.</t>
+          <t>Escluso dalla Coppa per precauzione (ginocchio), zero minuti stagionali: non è un investimento.</t>
         </is>
       </c>
     </row>
@@ -18088,7 +18264,7 @@
       </c>
       <c r="J70" s="36" t="inlineStr">
         <is>
-          <t>PSG concreto ma LUI vuole restare: rischio 'resta e non gioca' immutato (75/25 per Kolo Muani). Lasciarlo.</t>
+          <t>IN USCITA vera: PSG e Aston Villa, la Juve non si oppone (sblocca Zirkzee). Lasciarlo.</t>
         </is>
       </c>
     </row>
@@ -18132,7 +18308,7 @@
       </c>
       <c r="J71" s="41" t="inlineStr">
         <is>
-          <t>Diventa il 9 solo se Pinamonti parte davvero (trattativa rallentata): scommessa condizionata, verificare al 1/9.</t>
+          <t>TRIGGER QUASI SCATTATO: è il 9 nella probabile di Coppa con Pinamonti fuori per mercato. Se Pinamonti-Lazio chiude entro il 23/8, parte titolare alla 1ª.</t>
         </is>
       </c>
     </row>
@@ -18262,7 +18438,7 @@
       </c>
       <c r="F76" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>FUORI dall'XI di Coppa</t>
         </is>
       </c>
       <c r="G76" s="35" t="inlineStr">
@@ -18276,11 +18452,11 @@
         </is>
       </c>
       <c r="I76" s="10" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="J76" s="36" t="inlineStr">
         <is>
-          <t>Titolare nel 4-3-3 confermato ma BRUCIATO (2 TOP del Frosinone per FantaMaster): budget su.</t>
+          <t>ALLARME: non era nell'XI di Coppa (tridente Kvernadze-Raimondo-FINI). Da titolare bruciato a ballottaggio: dimezzare il tetto.</t>
         </is>
       </c>
     </row>
@@ -18334,41 +18510,41 @@
       </c>
       <c r="B78" s="43" t="inlineStr">
         <is>
-          <t>Maldini</t>
+          <t>Kvernadze</t>
         </is>
       </c>
       <c r="C78" s="35" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D78" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F78" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G78" s="35" t="inlineStr">
         <is>
-          <t>Conteso con Kevin Carlos</t>
+          <t>No (3° sui piazzati)</t>
         </is>
       </c>
       <c r="H78" s="36" t="inlineStr">
         <is>
-          <t>Titolarissimo a Cagliari</t>
+          <t>Ha vinto il ballottaggio nel tridente</t>
         </is>
       </c>
       <c r="I78" s="10" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J78" s="36" t="inlineStr">
         <is>
-          <t>Titolare in 7/7 fonti — la certezza del Cagliari — ma rigori CONTESI (Fantacalcio.it dà Kevin Carlos): pagare titolarità + punizioni, il premio rigori a metà.</t>
+          <t>PROMOSSO DAL CAMPO: titolare nel tridente di Coppa (16/8) con Raimondo e Fini — Schmid e Ghedjemis fuori. Qt 4: comprare prima che se ne accorgano.</t>
         </is>
       </c>
     </row>
@@ -18378,41 +18554,41 @@
       </c>
       <c r="B79" s="38" t="inlineStr">
         <is>
-          <t>Tourè E.</t>
+          <t>Maldini</t>
         </is>
       </c>
       <c r="C79" s="39" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D79" s="40" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E79" s="40" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="F79" s="39" t="inlineStr">
         <is>
-          <t>Titolare e rigorista</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G79" s="39" t="inlineStr">
         <is>
-          <t>Sì (3/3)</t>
+          <t>No (Deiola dal campo)</t>
         </is>
       </c>
       <c r="H79" s="41" t="inlineStr">
         <is>
-          <t>Il 9 del Parma dopo Pellegrino</t>
+          <t>Titolarissimo a Cagliari</t>
         </is>
       </c>
       <c r="I79" s="40" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="J79" s="41" t="inlineStr">
         <is>
-          <t>Il 9 del Parma con Pellegrino ufficialmente partito: rigori (3/3) e posto. Alzare il tetto.</t>
+          <t>Panchina all'esordio in Coppa (dentro al 54') e rigori a Deiola sul campo; FVM intanto salito a 22. Pagare solo la titolarità attesa.</t>
         </is>
       </c>
     </row>
@@ -18422,41 +18598,41 @@
       </c>
       <c r="B80" s="43" t="inlineStr">
         <is>
-          <t>Camarda</t>
+          <t>Tourè E.</t>
         </is>
       </c>
       <c r="C80" s="35" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D80" s="10" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="F80" s="35" t="inlineStr">
         <is>
-          <t>Alta (rotazioni)</t>
+          <t>Titolare e rigorista</t>
         </is>
       </c>
       <c r="G80" s="35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sì (3/3)</t>
         </is>
       </c>
       <c r="H80" s="36" t="inlineStr">
         <is>
-          <t>Il talento più atteso</t>
+          <t>Il 9 del Parma dopo Pellegrino</t>
         </is>
       </c>
       <c r="I80" s="10" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="J80" s="36" t="inlineStr">
         <is>
-          <t>Nel Milan avrà il suo spazio: colpo in prospettiva</t>
+          <t>Il 9 del Parma con Pellegrino ufficialmente partito: rigori (3/3) e posto. Alzare il tetto.</t>
         </is>
       </c>
     </row>
@@ -18466,23 +18642,23 @@
       </c>
       <c r="B81" s="38" t="inlineStr">
         <is>
-          <t>Boga</t>
+          <t>Camarda</t>
         </is>
       </c>
       <c r="C81" s="39" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D81" s="40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E81" s="40" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F81" s="39" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Alta (rotazioni)</t>
         </is>
       </c>
       <c r="G81" s="39" t="inlineStr">
@@ -18492,7 +18668,7 @@
       </c>
       <c r="H81" s="41" t="inlineStr">
         <is>
-          <t>Da schierare a prescindere</t>
+          <t>Il talento più atteso</t>
         </is>
       </c>
       <c r="I81" s="40" t="n">
@@ -18500,7 +18676,7 @@
       </c>
       <c r="J81" s="41" t="inlineStr">
         <is>
-          <t>Alla Juventus da jolly offensivo (W;A)</t>
+          <t>Nel Milan avrà il suo spazio: colpo in prospettiva</t>
         </is>
       </c>
     </row>
@@ -18510,23 +18686,23 @@
       </c>
       <c r="B82" s="43" t="inlineStr">
         <is>
-          <t>Raimondo</t>
+          <t>Boga</t>
         </is>
       </c>
       <c r="C82" s="35" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D82" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E82" s="10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F82" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Ballottaggio</t>
         </is>
       </c>
       <c r="G82" s="35" t="inlineStr">
@@ -18536,15 +18712,15 @@
       </c>
       <c r="H82" s="36" t="inlineStr">
         <is>
-          <t>11 gol in B, 3° marcatore tra le promosse</t>
+          <t>Da schierare a prescindere</t>
         </is>
       </c>
       <c r="I82" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J82" s="36" t="inlineStr">
         <is>
-          <t>Punta centrale del 4-3-3 ciociaro, riscattata dal Bologna.</t>
+          <t>Alla Juventus da jolly offensivo (W;A)</t>
         </is>
       </c>
     </row>
@@ -18554,41 +18730,41 @@
       </c>
       <c r="B83" s="38" t="inlineStr">
         <is>
-          <t>Rrahmani Al.</t>
+          <t>Raimondo</t>
         </is>
       </c>
       <c r="C83" s="39" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D83" s="40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E83" s="40" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F83" s="39" t="inlineStr">
         <is>
-          <t>3ª opzione (30%)</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G83" s="39" t="inlineStr">
         <is>
-          <t>In alternanza con Adams</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H83" s="41" t="inlineStr">
         <is>
-          <t>15 gol con lo Sparta Praga</t>
+          <t>11 gol in B, 3° marcatore tra le promosse</t>
         </is>
       </c>
       <c r="I83" s="40" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J83" s="41" t="inlineStr">
         <is>
-          <t>In alternanza-rigori con Adams e 3ª punta nelle gerarchie: ultimo slot con upside vero.</t>
+          <t>Titolare in Coppa (16/8): confermato dal campo.</t>
         </is>
       </c>
     </row>
@@ -18598,41 +18774,41 @@
       </c>
       <c r="B84" s="43" t="inlineStr">
         <is>
-          <t>Geubbels</t>
+          <t>Rrahmani Al.</t>
         </is>
       </c>
       <c r="C84" s="35" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D84" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E84" s="10" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F84" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>3ª opzione (30%)</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>In alternanza con Adams</t>
         </is>
       </c>
       <c r="H84" s="36" t="inlineStr">
         <is>
-          <t>Fisicità nel Lecce</t>
+          <t>15 gol con lo Sparta Praga</t>
         </is>
       </c>
       <c r="I84" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J84" s="36" t="inlineStr">
         <is>
-          <t>Confermato 70/30 su Stulic, 7/7 dal dischetto: oro semi-noto.</t>
+          <t>Subentro al 74' in Coppa: resta l'alternanza-rigori con Adams. Ultimo slot con upside.</t>
         </is>
       </c>
     </row>
@@ -18642,33 +18818,33 @@
       </c>
       <c r="B85" s="38" t="inlineStr">
         <is>
-          <t>Piccoli</t>
+          <t>Geubbels</t>
         </is>
       </c>
       <c r="C85" s="39" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D85" s="40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E85" s="40" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F85" s="39" t="inlineStr">
         <is>
-          <t>Alta (rotazioni)</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G85" s="39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Conteso (fonti spaccate)</t>
         </is>
       </c>
       <c r="H85" s="41" t="inlineStr">
         <is>
-          <t>Vice Kean di lusso</t>
+          <t>Fisicità nel Lecce</t>
         </is>
       </c>
       <c r="I85" s="40" t="n">
@@ -18676,7 +18852,7 @@
       </c>
       <c r="J85" s="41" t="inlineStr">
         <is>
-          <t>UFFICIALE al Bologna ma è il VICE-Dovbyk (30%), non trequartista: non pagarlo da titolare.</t>
+          <t>Favorito per il POSTO (Stulic fuori dalla probabile) ma i rigori non sono più un dato pacifico (4 fonti su 7 dicono Stulic). Palermo-Lecce 17/8 da guardare.</t>
         </is>
       </c>
     </row>
@@ -18686,23 +18862,23 @@
       </c>
       <c r="B86" s="43" t="inlineStr">
         <is>
-          <t>Ratkov</t>
+          <t>Piccoli</t>
         </is>
       </c>
       <c r="C86" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D86" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F86" s="35" t="inlineStr">
         <is>
-          <t>Conteso a 3 + mercato</t>
+          <t>Alta (rotazioni)</t>
         </is>
       </c>
       <c r="G86" s="35" t="inlineStr">
@@ -18712,7 +18888,7 @@
       </c>
       <c r="H86" s="36" t="inlineStr">
         <is>
-          <t>Grande precampionato</t>
+          <t>Vice Kean di lusso</t>
         </is>
       </c>
       <c r="I86" s="10" t="n">
@@ -18720,7 +18896,7 @@
       </c>
       <c r="J86" s="36" t="inlineStr">
         <is>
-          <t>EVITARE: posto conteso a tre (Ratkov/Dia/Noslin 40/30/30) e club che vuole cederlo (Dynamo Mosca).</t>
+          <t>UFFICIALE al Bologna ma è il VICE-Dovbyk (30%), non trequartista: non pagarlo da titolare.</t>
         </is>
       </c>
     </row>
@@ -18730,23 +18906,23 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Mendy P.</t>
+          <t>Ratkov</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E87" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Conteso a 3 + mercato</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -18756,15 +18932,15 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Possibile sorpresa</t>
+          <t>Grande precampionato</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>BRUCIATO (Calcio d'Angolo a 1 credito): la doppietta all'Atalanta l'hanno vista tutti.</t>
+          <t>EVITARE: posto conteso a tre (Ratkov/Dia/Noslin 40/30/30) e club che vuole cederlo (Dynamo Mosca).</t>
         </is>
       </c>
     </row>
@@ -18774,19 +18950,19 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Ekhator</t>
+          <t>Mendy P.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E88" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -18800,15 +18976,15 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Prospettiva Juve</t>
+          <t>Possibile sorpresa</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Bicipite femorale ko, punta la 1ª: sorpresa da subentro dietro Kolo Muani (FantaMaster). Ultimo slot.</t>
+          <t>PROMOSSO: titolare in Coppa (Kevin Carlos assente): la scommessa a 2-3 si rafforza.</t>
         </is>
       </c>
     </row>
@@ -18818,39 +18994,83 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>Ekhator</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>3</v>
+      </c>
+      <c r="E89" t="n">
+        <v>10</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Prospettiva Juve</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>4</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Bicipite femorale ko, punta la 1ª: sorpresa da subentro dietro Kolo Muani (FantaMaster). Ultimo slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>15</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>Noslin</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Lazio</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D90" t="n">
         <v>6</v>
       </c>
-      <c r="E89" t="n">
+      <c r="E90" t="n">
         <v>17</v>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>Ballottaggio</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G90" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H90" t="inlineStr">
         <is>
           <t>Jolly offensivo Lazio</t>
         </is>
       </c>
-      <c r="I89" t="n">
+      <c r="I90" t="n">
         <v>5</v>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="J90" t="inlineStr">
         <is>
           <t>In corsa a tre per il posto da 9 della Lazio (Goal/Calciodangolo lo danno titolare): scommessa da 1-3 crediti.</t>
         </is>

</xml_diff>

<commit_message>
chore(wishlist): bake 76 morning ops into asta.xlsx, ops emptied (v1.3.0)
Full-rewrite of the 4 role sheets, object-equivalence check OK, prio-1
unchanged in every slot (Asta sheet already aligned), 4 charts intact.
New wishlist entries: Mascardi (P3), Doig (D7), Comuzzo/Marcandalli (D8),
Cichella (C8), Borrelli/Havel (A6). Smoke test 66 assert PASS.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asta.xlsx
+++ b/asta.xlsx
@@ -4063,7 +4063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="F10" s="35" t="inlineStr">
         <is>
-          <t>Ballottaggio 50/50 (conflitto fonti)</t>
+          <t>Ballottaggio 50/50 (fonti Milan: Torriani avanti)</t>
         </is>
       </c>
       <c r="G10" s="35" t="inlineStr">
@@ -4361,11 +4361,11 @@
         </is>
       </c>
       <c r="I10" s="10" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J10" s="36" t="inlineStr">
         <is>
-          <t>CONFLITTO: porte dà Maignan 65-70%, probabili dà Torriani 60-65 (Maignan rientrato solo il 15-16/8, zero precampionato). Non pagare la porta Milan da titolare certo</t>
+          <t>Rientrato solo il 16/8, 6 giorni al Toro; Amorim lo vorrebbe ma decidono i test. Probabili definitive DOPO l'asta. E il Milan alla 1ª rischia senza Pulisic, Gimenez e Leao: Torriani copertura a 1</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Titolare (RESTA al Lecce)</t>
+          <t>Titolare MA in pole come vice-Meret al Napoli</t>
         </is>
       </c>
       <c r="G20" s="35" t="inlineStr">
@@ -4728,11 +4728,11 @@
         </is>
       </c>
       <c r="I20" s="10" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="J20" s="36" t="inlineStr">
         <is>
-          <t>RESTA e diventa CAPITANO (Fruchtl al Salisburgo); voce-Napoli fredda (vanno su Restes). MV 6,4: semi-bruciato</t>
+          <t>CalcioNapoli24 16/8: ha superato Kovar e Vicario per il ruolo di vice al Napoli; il presidente nega, lui è freddo, ma se parte va da riserva. Solo a sconto</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="F22" s="35" t="inlineStr">
         <is>
-          <t>Titolare (spalla da monitorare)</t>
+          <t>Titolare (90' il 15/8, spalla ok)</t>
         </is>
       </c>
       <c r="G22" s="35" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="J22" s="36" t="inlineStr">
         <is>
-          <t>Titolare in Coppa 15/8 ma staff cauto sulla spalla (preso Selvik); pianetafanta lo dava ancora ko. Ok senza strapagare</t>
+          <t>Cautela dello staff rientrata. CORREZIONE: Selvik NON è arrivato (va al Brest), il vice è Padelli</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Titolare (75-80%)</t>
+          <t>Titolare ~65% (rebus cessione)</t>
         </is>
       </c>
       <c r="G23" s="35" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="J23" s="36" t="inlineStr">
         <is>
-          <t>Riscattato; Turati RESTA come vice (Samp raffreddata). Test finale Sassuolo-Cesena 17/8. Bruciato dalle guide del 16/8</t>
+          <t>Riscattato MA ha dichiarato chiusa l'esperienza e il club valuta la cessione (SassuoloNews: 'l'erede è Turati'); probabili di stasera discordanti. Solo a sconto o in coppia con Turati</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="F28" s="35" t="inlineStr">
         <is>
-          <t>APERTO (mercato porta)</t>
+          <t>Titolare (piste esterne chiuse)</t>
         </is>
       </c>
       <c r="G28" s="35" t="inlineStr">
@@ -5080,11 +5080,11 @@
         </is>
       </c>
       <c r="I28" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J28" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO: il Monza cerca un portiere 'non semplice vice' (idee Montipò/Audero/Di Gregorio). Solo a 1-3</t>
+          <t>Titolare in Coppa (3-0 all'Avellino), Pizzignacco trattenuto, Montipò al Venezia e Di Gregorio verso il Valencia: il rischio mister-X si è sgonfiato</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="F32" s="35" t="inlineStr">
         <is>
-          <t>Titolare 1ª (80-85%)</t>
+          <t>Titolare 1ª (85-90%) ma a scadenza</t>
         </is>
       </c>
       <c r="G32" s="35" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="J32" s="36" t="inlineStr">
         <is>
-          <t>Spalletti: 'stavolta gioca Perin'. Upside reale finché la Juve non chiude Dibu/Vicario: chiamata da 2-3 con margine</t>
+          <t>Spalletti: 'stavolta gioca Perin'. Dibu SCARTATO, arriva VICARIO (chiusura 24-72h): dalla 2ª-3ª la porta è sua. Vale le primissime giornate</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>In uscita (proposto Juve)</t>
+          <t>In uscita (Hull City, stallo formula)</t>
         </is>
       </c>
       <c r="G35" s="35" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="F36" s="35" t="inlineStr">
         <is>
-          <t>Titolare (65-70%)</t>
+          <t>Titolare (70%)</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="J36" s="36" t="inlineStr">
         <is>
-          <t>Titolare e clean sheet nel 3-0 del 16/8; elogi di Alvini. Nessuna guida lo cita: il P-scommessa migliore</t>
+          <t>CORREZIONE: il 16/8 è finita 4-1 e HA SUBITO GOL (niente clean sheet). Resta avanti su Desplanches ma FantaMaster mette entrambi tra i flop: 2-3 senza hype</t>
         </is>
       </c>
     </row>
@@ -5373,23 +5373,23 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Turati</t>
+          <t>Mascardi</t>
         </is>
       </c>
       <c r="C37" s="35" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D37" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Copertura a costo zero</t>
         </is>
       </c>
       <c r="G37" s="35" t="inlineStr">
@@ -5399,15 +5399,15 @@
       </c>
       <c r="H37" s="36" t="inlineStr">
         <is>
-          <t>Possibile rilancio</t>
+          <t>Titolare in Coppa (1-0 alla Carrarese)</t>
         </is>
       </c>
       <c r="I37" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J37" s="36" t="inlineStr">
         <is>
-          <t>Non più in uscita (Samp raffreddata): resta il vice di Muric. Da 1 come copertura</t>
+          <t>Perri è fatta (visite oggi) ma NON listato e con zero precampionato: se la porta Toro non è copribile, Mascardi a 1 è la scommessa asimmetrica. Paleari in uscita</t>
         </is>
       </c>
     </row>
@@ -5417,23 +5417,23 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Sportiello</t>
+          <t>Turati</t>
         </is>
       </c>
       <c r="C38" s="35" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D38" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F38" s="35" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -5443,15 +5443,15 @@
       </c>
       <c r="H38" s="36" t="inlineStr">
         <is>
-          <t>Vice affidabile</t>
+          <t>Possibile rilancio</t>
         </is>
       </c>
       <c r="I38" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J38" s="36" t="inlineStr">
         <is>
-          <t>Vice Carnesecchi: copertura per chi ha il titolare Atalanta</t>
+          <t>Non più in uscita (Samp raffreddata): resta il vice di Muric. Da 1 come copertura</t>
         </is>
       </c>
     </row>
@@ -5461,23 +5461,23 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Daffara</t>
+          <t>Sportiello</t>
         </is>
       </c>
       <c r="C39" s="35" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D39" s="10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Infortunato (rientro 2ª)</t>
+          <t>Bassa</t>
         </is>
       </c>
       <c r="G39" s="35" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="H39" s="36" t="inlineStr">
         <is>
-          <t>Jolly Parma</t>
+          <t>Vice affidabile</t>
         </is>
       </c>
       <c r="I39" s="10" t="n">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="J39" s="36" t="inlineStr">
         <is>
-          <t>Lesione di basso grado alla coscia destra: salta la 1ª. Da 1 solo per l'alternanza futura</t>
+          <t>Vice Carnesecchi: copertura per chi ha il titolare Atalanta</t>
         </is>
       </c>
     </row>
@@ -5505,23 +5505,23 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Motta</t>
+          <t>Daffara</t>
         </is>
       </c>
       <c r="C40" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D40" s="10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F40" s="35" t="inlineStr">
         <is>
-          <t>Vice Mandas</t>
+          <t>Infortunato (rientro 2ª)</t>
         </is>
       </c>
       <c r="G40" s="35" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="H40" s="36" t="inlineStr">
         <is>
-          <t>Vicino in gerarchia (SOS)</t>
+          <t>Jolly Parma</t>
         </is>
       </c>
       <c r="I40" s="10" t="n">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="J40" s="36" t="inlineStr">
         <is>
-          <t>A 1 credito: la coppia Mandas+Motta è il ponte-porta consigliato da SOS. Provedel ceduto all'Inter.</t>
+          <t>Lesione di basso grado alla coscia destra: salta la 1ª. Da 1 solo per l'alternanza futura</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Terracciano</t>
+          <t>Motta</t>
         </is>
       </c>
       <c r="C41" s="35" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D41" s="10" t="n">
@@ -5565,7 +5565,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Vice Mandas</t>
         </is>
       </c>
       <c r="G41" s="35" t="inlineStr">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="H41" s="36" t="inlineStr">
         <is>
-          <t>Vice Maignan</t>
+          <t>Vicino in gerarchia (SOS)</t>
         </is>
       </c>
       <c r="I41" s="10" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="J41" s="36" t="inlineStr">
         <is>
-          <t>Copertura per chi ha il titolare Milan</t>
+          <t>A 1 credito: la coppia Mandas+Motta è il ponte-porta consigliato da SOS. Provedel ceduto all'Inter.</t>
         </is>
       </c>
     </row>
@@ -5593,12 +5593,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Sherri</t>
+          <t>Terracciano</t>
         </is>
       </c>
       <c r="C42" s="35" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="H42" s="36" t="inlineStr">
         <is>
-          <t>Vice Caprile</t>
+          <t>Vice Maignan</t>
         </is>
       </c>
       <c r="I42" s="10" t="n">
@@ -5627,14 +5627,58 @@
       </c>
       <c r="J42" s="36" t="inlineStr">
         <is>
+          <t>Copertura per chi ha il titolare Milan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Sherri</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="35" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="G43" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="36" t="inlineStr">
+        <is>
+          <t>Vice Caprile</t>
+        </is>
+      </c>
+      <c r="I43" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" s="36" t="inlineStr">
+        <is>
           <t>Copertura Cagliari</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A30:J30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5648,7 +5692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5818,7 +5862,7 @@
       </c>
       <c r="J7" s="36" t="inlineStr">
         <is>
-          <t>Distorsione caviglia LIEVE: punta la 1ª da titolare (a sinistra). Allarme fairplay RIDOTTO: fonti fresche parlano di 4 gialli in 11 in miglioramento</t>
+          <t>CORREZIONE DI LATO: gioca a SINISTRA (Molina a destra). Distorsione lieve, ~80% alla 1ª (lunedì 24/8: 10 giorni di recupero)</t>
         </is>
       </c>
     </row>
@@ -6317,7 +6361,7 @@
       </c>
       <c r="J20" s="36" t="inlineStr">
         <is>
-          <t>Titolare certo MA 2 espulsioni + 6 gialli nel 25/26: col bonus fairplay il malus pesa doppio.</t>
+          <t>CORREZIONE DI LATO: gioca a SINISTRA (Molina a destra). Distorsione lieve, ~80% alla 1ª</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6475,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Entra al 60' (Bellanova avanti)</t>
+          <t>Terzino nel 4-3-3 di Sarri: 50/50 con Bellanova</t>
         </is>
       </c>
       <c r="G23" s="35" t="inlineStr">
@@ -6445,11 +6489,11 @@
         </is>
       </c>
       <c r="I23" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J23" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO dal campo: al Bortolotti è entrato per Bellanova, che è il quinto destro di Sarri</t>
+          <t>Sarri è passato alla difesa a 4: non più quinti, ballottaggio vero</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6519,7 @@
       </c>
       <c r="F24" s="35" t="inlineStr">
         <is>
-          <t>IN USCITA (Nottingham Forest)</t>
+          <t>RESTA (rinnovo-ponte) ma panchina in Coppa</t>
         </is>
       </c>
       <c r="G24" s="35" t="inlineStr">
@@ -6489,11 +6533,11 @@
         </is>
       </c>
       <c r="I24" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J24" s="36" t="inlineStr">
         <is>
-          <t>Cessione 'concordata' per il filone probabili (vs rinnovo-ponte per il filone mercato: conflitto). In campo Jimenez 55/Joao Mario 45: non comprarlo</t>
+          <t>TMW 12/8: inversione, si valuta rinnovo annuale, nessuna offerta Forest. Ma col Benevento ha giocato Joao Mario: destra contesa a 3-4</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6739,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Terzino nel 4-3-3: 50/50 con Zappacosta</t>
         </is>
       </c>
       <c r="G29" s="35" t="inlineStr">
@@ -6709,11 +6753,11 @@
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J29" s="36" t="inlineStr">
         <is>
-          <t>Titolare con Sarri (davanti a Zappacosta). Offerta formale Fulham 20M RESPINTA ('incedibile') ma pressing inglese fino all'1/9</t>
+          <t>Nel 4-3-3 il posto non è più blindato + Fulham respinto ma colloqui aperti (Romano 16/8)</t>
         </is>
       </c>
     </row>
@@ -7194,7 +7238,7 @@
       </c>
       <c r="F42" s="35" t="inlineStr">
         <is>
-          <t>APERTO (conflitto fonti)</t>
+          <t>Titolare atteso (recuperato)</t>
         </is>
       </c>
       <c r="G42" s="35" t="inlineStr">
@@ -7212,7 +7256,7 @@
       </c>
       <c r="J42" s="36" t="inlineStr">
         <is>
-          <t>CONFLITTO: entrato col Man United il 15/8 vs pianetafanta/SOS che segnalano lesione al retto femorale. Verificare prima dell'asta</t>
+          <t>RISOLTO: esami negativi, entrato col Man United il 15/8, Gazzetta lo dà titolare col Torino. Braccetto sinistro di Amorim (~75-85%)</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7429,7 @@
       </c>
       <c r="F48" s="35" t="inlineStr">
         <is>
-          <t>Panchina il 16/8 (turnover?)</t>
+          <t>Titolare atteso (panchina 16/8 = turnover)</t>
         </is>
       </c>
       <c r="G48" s="35" t="inlineStr">
@@ -7403,7 +7447,7 @@
       </c>
       <c r="J48" s="36" t="inlineStr">
         <is>
-          <t>FRENATO: in panchina con l'Ascoli (terzetto Marcandalli-Otoa-Vasquez). Ex designato sui rigori e 5 gol, ma il 'promosso' va congelato fino all'XI col Napoli: 8-12 max</t>
+          <t>Entrato al 46' con l'Ascoli, tutte le tipo lo danno titolare. L'episodio-rigore con Colombo è di APRILE: peso ridotto. Restano i 7 gialli</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7693,7 @@
       </c>
       <c r="F54" s="35" t="inlineStr">
         <is>
-          <t>Risalito (amichevoli 16/8)</t>
+          <t>Ridimensionato: Chalobah recuperato</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
@@ -7663,11 +7707,11 @@
         </is>
       </c>
       <c r="I54" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J54" s="36" t="inlineStr">
         <is>
-          <t>Ha giocato ENTRAMBE le amichevoli col Liverpool mentre Chalobah nessuna: il declassamento era prematuro. 3-4</t>
+          <t>Chalobah 84' ad Anfield il 16/8: il suo declassamento era un errore. Kempf torna alternativa</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7825,7 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Titolare (buco Lucumì)</t>
+          <t>Titolare (con Heggem)</t>
         </is>
       </c>
       <c r="G57" s="35" t="inlineStr">
@@ -7799,7 +7843,7 @@
       </c>
       <c r="J57" s="36" t="inlineStr">
         <is>
-          <t>Con Lucumì alla Juve (visite 16/8) e Casale ko la coppia è Vitik-Heggem; titolare nella formazione-tipo. Un report SOS del 6/8 segnalava un affaticamento: verificare</t>
+          <t>RIABILITATO dalle probabili aggiornate (Helland alternativa). Occhio all'arrivo di Cabal dalla Juve (in chiusura)</t>
         </is>
       </c>
     </row>
@@ -7825,7 +7869,7 @@
       </c>
       <c r="F58" s="35" t="inlineStr">
         <is>
-          <t>APERTO (assente il 16/8)</t>
+          <t>Titolare (84' ad Anfield il 16/8)</t>
         </is>
       </c>
       <c r="G58" s="35" t="inlineStr">
@@ -7839,11 +7883,11 @@
         </is>
       </c>
       <c r="I58" s="10" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J58" s="36" t="inlineStr">
         <is>
-          <t>FRENATO: fuori da entrambe le amichevoli col Liverpool, motivo non verificabile — da richiudere prima del 22/8. Le guide lo danno titolare certo: non fidarsi a prezzo pieno</t>
+          <t>GIALLO RISOLTO: nessun infortunio, titolare col Liverpool, Fabregas lo elogia. ~85-95% alla 1ª: torna comprabile da titolare</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8369,7 @@
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Ballottaggio (~50/50)</t>
+          <t>Favorito 60/40 (Holm recuperato)</t>
         </is>
       </c>
       <c r="G71" s="35" t="inlineStr">
@@ -8343,7 +8387,7 @@
       </c>
       <c r="J71" s="36" t="inlineStr">
         <is>
-          <t>Holm recuperato (37' col Pisa + Brighton) punta la 1ª da titolare: il 70/30 non regge più.</t>
+          <t>Holm rientrato (72' col Brighton, punta la 1ª) ma Zortea resta avanti nella tipo di Tedesco</t>
         </is>
       </c>
     </row>
@@ -8413,7 +8457,7 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Risalito (50/50 con Kaiki)</t>
+          <t>Ridimensionato: Kaiki favorito</t>
         </is>
       </c>
       <c r="G73" s="35" t="inlineStr">
@@ -8427,11 +8471,11 @@
         </is>
       </c>
       <c r="I73" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J73" s="36" t="inlineStr">
         <is>
-          <t>Titolare in ENTRAMBE le amichevoli col Liverpool del 16/8 (Kaiki in nessuna): il ballottaggio si è riaperto del tutto</t>
+          <t>CORREZIONE: col Liverpool Valle è SUBENTRATO al 35' per Kaiki. Kaiki 60/Valle 40</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8868,7 @@
       </c>
       <c r="F84" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Ridimensionato: Kaiki favorito</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -8838,11 +8882,11 @@
         </is>
       </c>
       <c r="I84" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J84" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come D5</t>
+          <t>CORREZIONE: col Liverpool è subentrato al 35' per Kaiki. Kaiki 60/Valle 40</t>
         </is>
       </c>
     </row>
@@ -9044,7 +9088,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Risalito (tipo)</t>
+          <t>Panchina il 15/8 (Hainaut avanti)</t>
         </is>
       </c>
       <c r="G89" s="35" t="inlineStr">
@@ -9058,7 +9102,7 @@
         </is>
       </c>
       <c r="I89" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J89" s="36" t="inlineStr">
         <is>
@@ -9279,7 +9323,7 @@
       </c>
       <c r="F96" s="35" t="inlineStr">
         <is>
-          <t>Titolare (campo)</t>
+          <t>Titolare (campo 15/8; Sverko out)</t>
         </is>
       </c>
       <c r="G96" s="35" t="inlineStr">
@@ -9293,11 +9337,11 @@
         </is>
       </c>
       <c r="I96" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J96" s="36" t="inlineStr">
         <is>
-          <t>Titolare in Coppa ma il tipo dà Moreno terzo centrale: conflitto aperto. 2-3 max</t>
+          <t>Conflitto RISOLTO A FAVORE: titolare col Modena al posto di Moreno, e Sverko è out fino a ottobre. Semi-bruciato (Lottomatica)</t>
         </is>
       </c>
     </row>
@@ -9323,7 +9367,7 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Titolare (campo)</t>
+          <t>Titolare (campo 15/8, Correia panchina)</t>
         </is>
       </c>
       <c r="G97" s="35" t="inlineStr">
@@ -9341,7 +9385,7 @@
       </c>
       <c r="J97" s="36" t="inlineStr">
         <is>
-          <t>Titolare in Coppa ma nel tipo il quinto destro è Correia: conflitto aperto. 2-3 max</t>
+          <t>Conflitto risolto a favore: il quinto destro è lui</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9465,7 @@
       </c>
       <c r="H99" s="36" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Titolare 90' il 16/8</t>
         </is>
       </c>
       <c r="I99" s="10" t="n">
@@ -9429,7 +9473,7 @@
       </c>
       <c r="J99" s="36" t="inlineStr">
         <is>
-          <t>PROMOSSO: terzino/braccetto titolare e GOL in Coppa il 16/8, davanti a Bracaglia nell'XI reale</t>
+          <t>CORREZIONE: NESSUN gol suo il 16/8 (marcatori: Kvernadze x2, Cichella, Raimondo). Resta titolare e non citato dalle guide</t>
         </is>
       </c>
     </row>
@@ -9439,7 +9483,7 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Obrador</t>
+          <t>Doig</t>
         </is>
       </c>
       <c r="C100" s="35" t="inlineStr">
@@ -9448,14 +9492,14 @@
         </is>
       </c>
       <c r="D100" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E100" s="10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F100" s="35" t="inlineStr">
         <is>
-          <t>Titolare (tipo)</t>
+          <t>Titolare (65/35 su Obrador)</t>
         </is>
       </c>
       <c r="G100" s="35" t="inlineStr">
@@ -9465,15 +9509,15 @@
       </c>
       <c r="H100" s="36" t="inlineStr">
         <is>
-          <t>Fascia sinistra del Sassuolo</t>
+          <t>Fascia sinistra nel 4-3-3 di Aquilani</t>
         </is>
       </c>
       <c r="I100" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J100" s="36" t="inlineStr">
         <is>
-          <t>Nella formazione-tipo del 16/8 la fascia sinistra è SUA (Doig fuori): quadro ribaltato in una settimana</t>
+          <t>RIABILITATO: titolare nelle probabili di stasera e nella tipo. Verificare l'XI delle 18:30 se l'asta lo consente</t>
         </is>
       </c>
     </row>
@@ -9483,23 +9527,23 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Kaiki</t>
+          <t>Obrador</t>
         </is>
       </c>
       <c r="C101" s="35" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D101" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E101" s="10" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Superato: Doig titolare</t>
         </is>
       </c>
       <c r="G101" s="35" t="inlineStr">
@@ -9509,15 +9553,15 @@
       </c>
       <c r="H101" s="36" t="inlineStr">
         <is>
-          <t>5 assist nel 2025 da terzino</t>
+          <t>Fascia sinistra del Sassuolo</t>
         </is>
       </c>
       <c r="I101" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J101" s="36" t="inlineStr">
         <is>
-          <t>RISCHIO AL RIBASSO: Valle titolare in entrambe le amichevoli del 16/8, lui in nessuna — e le guide lo hanno bruciato. 4-6 max</t>
+          <t>RIBALTONE-2: probabili del 17/8 e tipo di Aquilani danno Doig a sinistra ('Obrador arrivato tardi, poca integrazione')</t>
         </is>
       </c>
     </row>
@@ -9527,23 +9571,23 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Biraghi</t>
+          <t>Kaiki</t>
         </is>
       </c>
       <c r="C102" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D102" s="10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E102" s="10" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F102" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Tornato favorito (60/40 su Valle)</t>
         </is>
       </c>
       <c r="G102" s="35" t="inlineStr">
@@ -9553,15 +9597,15 @@
       </c>
       <c r="H102" s="36" t="inlineStr">
         <is>
-          <t>Tutti i piazzati del Torino</t>
+          <t>5 assist nel 2025 da terzino</t>
         </is>
       </c>
       <c r="I102" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J102" s="36" t="inlineStr">
         <is>
-          <t>Una stagione intera da titolare può riportarlo ad alti livelli</t>
+          <t>Il campo del 16/8 lo rimette avanti; resta bruciato (Sisal): 4-6 max</t>
         </is>
       </c>
     </row>
@@ -9571,19 +9615,19 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Jimenez A.</t>
+          <t>Biraghi</t>
         </is>
       </c>
       <c r="C103" s="35" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D103" s="10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E103" s="10" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
@@ -9597,15 +9641,15 @@
       </c>
       <c r="H103" s="36" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Tutti i piazzati del Torino</t>
         </is>
       </c>
       <c r="I103" s="10" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J103" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come D6</t>
+          <t>Una stagione intera da titolare può riportarlo ad alti livelli</t>
         </is>
       </c>
     </row>
@@ -9615,19 +9659,19 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Norton-Cuffy</t>
+          <t>Jimenez A.</t>
         </is>
       </c>
       <c r="C104" s="35" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D104" s="10" t="n">
         <v>8</v>
       </c>
       <c r="E104" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F104" s="35" t="inlineStr">
         <is>
@@ -9641,15 +9685,15 @@
       </c>
       <c r="H104" s="36" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="I104" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J104" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come D5</t>
+          <t>Se non preso come D6</t>
         </is>
       </c>
     </row>
@@ -9659,23 +9703,23 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Monterisi</t>
+          <t>Norton-Cuffy</t>
         </is>
       </c>
       <c r="C105" s="35" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D105" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E105" s="10" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F105" s="35" t="inlineStr">
         <is>
-          <t>Titolare (campo)</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G105" s="35" t="inlineStr">
@@ -9685,15 +9729,15 @@
       </c>
       <c r="H105" s="36" t="inlineStr">
         <is>
-          <t>5 assist in B, sale sui piazzati</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="I105" s="10" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J105" s="36" t="inlineStr">
         <is>
-          <t>Titolare e perno anche nel 3-0 del 16/8 (clean sheet): confermato, sale sui piazzati</t>
+          <t>Se non preso come D5</t>
         </is>
       </c>
     </row>
@@ -9703,23 +9747,23 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Perez M.</t>
+          <t>Monterisi</t>
         </is>
       </c>
       <c r="C106" s="35" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D106" s="10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E106" s="10" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F106" s="35" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G106" s="35" t="inlineStr">
@@ -9729,15 +9773,15 @@
       </c>
       <c r="H106" s="36" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>5 assist in B, sale sui piazzati</t>
         </is>
       </c>
       <c r="I106" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J106" s="36" t="inlineStr">
         <is>
-          <t>Tappabuchi a 1</t>
+          <t>Titolare e perno anche nel 3-0 del 16/8 (clean sheet): confermato, sale sui piazzati</t>
         </is>
       </c>
     </row>
@@ -9747,23 +9791,23 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>Kempf</t>
+          <t>Perez M.</t>
         </is>
       </c>
       <c r="C107" s="35" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D107" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E107" s="10" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F107" s="35" t="inlineStr">
         <is>
-          <t>Fuori dall'XI atteso</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G107" s="35" t="inlineStr">
@@ -9773,15 +9817,15 @@
       </c>
       <c r="H107" s="36" t="inlineStr">
         <is>
-          <t>CS Como</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="I107" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J107" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO: l'XI atteso del Como dà Chalobah-Ramon centrali. Solo a 1-2 da copertura.</t>
+          <t>Tappabuchi a 1</t>
         </is>
       </c>
     </row>
@@ -9791,23 +9835,23 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>Tavares N.</t>
+          <t>Kempf</t>
         </is>
       </c>
       <c r="C108" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D108" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E108" s="10" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F108" s="35" t="inlineStr">
         <is>
-          <t>Ko ginocchio + ipotesi scambio</t>
+          <t>Fuori dall'XI atteso</t>
         </is>
       </c>
       <c r="G108" s="35" t="inlineStr">
@@ -9817,15 +9861,15 @@
       </c>
       <c r="H108" s="36" t="inlineStr">
         <is>
-          <t>Potenziale assist</t>
+          <t>CS Como</t>
         </is>
       </c>
       <c r="I108" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J108" s="36" t="inlineStr">
         <is>
-          <t>Infiammazione al ginocchio (fuori in Coppa, Pedraza titolare) e ipotesi scambio con Tomori: solo a saldo estremo.</t>
+          <t>DECLASSATO: l'XI atteso del Como dà Chalobah-Ramon centrali. Solo a 1-2 da copertura.</t>
         </is>
       </c>
     </row>
@@ -9835,23 +9879,23 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Correia T.</t>
+          <t>Tavares N.</t>
         </is>
       </c>
       <c r="C109" s="35" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D109" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E109" s="10" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F109" s="35" t="inlineStr">
         <is>
-          <t>Superato da Hainaut</t>
+          <t>Ko ginocchio + ipotesi scambio</t>
         </is>
       </c>
       <c r="G109" s="35" t="inlineStr">
@@ -9861,15 +9905,15 @@
       </c>
       <c r="H109" s="36" t="inlineStr">
         <is>
-          <t>Titolare Venezia</t>
+          <t>Potenziale assist</t>
         </is>
       </c>
       <c r="I109" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J109" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO DAL CAMPO: Hainaut titolare in Coppa, lui dentro al 74'. Solo ultimo slot.</t>
+          <t>Infiammazione al ginocchio (fuori in Coppa, Pedraza titolare) e ipotesi scambio con Tomori: solo a saldo estremo.</t>
         </is>
       </c>
     </row>
@@ -9879,170 +9923,170 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
+          <t>Correia T.</t>
+        </is>
+      </c>
+      <c r="C110" s="35" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E110" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F110" s="35" t="inlineStr">
+        <is>
+          <t>Superato da Hainaut</t>
+        </is>
+      </c>
+      <c r="G110" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H110" s="36" t="inlineStr">
+        <is>
+          <t>Titolare Venezia</t>
+        </is>
+      </c>
+      <c r="I110" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J110" s="36" t="inlineStr">
+        <is>
+          <t>DECLASSATO DAL CAMPO: Hainaut titolare in Coppa, lui dentro al 74'. Solo ultimo slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
           <t>Celik</t>
         </is>
       </c>
-      <c r="C110" s="35" t="inlineStr">
+      <c r="C111" s="35" t="inlineStr">
         <is>
           <t>Juventus</t>
         </is>
       </c>
-      <c r="D110" s="10" t="n">
+      <c r="D111" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E110" s="10" t="n">
+      <c r="E111" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="F110" s="35" t="inlineStr">
+      <c r="F111" s="35" t="inlineStr">
         <is>
           <t>Ballottaggio</t>
         </is>
       </c>
-      <c r="G110" s="35" t="inlineStr">
+      <c r="G111" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H110" s="36" t="inlineStr">
+      <c r="H111" s="36" t="inlineStr">
         <is>
           <t>Roma</t>
         </is>
       </c>
-      <c r="I110" s="10" t="n">
+      <c r="I111" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J110" s="36" t="inlineStr">
+      <c r="J111" s="36" t="inlineStr">
         <is>
           <t>Ora alla Juventus: in ballottaggio col favorito Kalulu (45/55) per la fascia destra. Non più titolare Roma.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="1" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
         <is>
           <t>SLOT D8 — Scommessa / parcheggio infortunati · budget consigliato: 3</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="44" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="44" t="inlineStr">
         <is>
           <t>Priorità</t>
         </is>
       </c>
-      <c r="B113" s="44" t="inlineStr">
+      <c r="B114" s="44" t="inlineStr">
         <is>
           <t>Giocatore</t>
         </is>
       </c>
-      <c r="C113" s="44" t="inlineStr">
+      <c r="C114" s="44" t="inlineStr">
         <is>
           <t>Squadra</t>
         </is>
       </c>
-      <c r="D113" s="44" t="inlineStr">
+      <c r="D114" s="44" t="inlineStr">
         <is>
           <t>Qt.A</t>
         </is>
       </c>
-      <c r="E113" s="44" t="inlineStr">
+      <c r="E114" s="44" t="inlineStr">
         <is>
           <t>FVM</t>
         </is>
       </c>
-      <c r="F113" s="44" t="inlineStr">
+      <c r="F114" s="44" t="inlineStr">
         <is>
           <t>Titolarità</t>
         </is>
       </c>
-      <c r="G113" s="44" t="inlineStr">
+      <c r="G114" s="44" t="inlineStr">
         <is>
           <t>Rigorista</t>
         </is>
       </c>
-      <c r="H113" s="44" t="inlineStr">
+      <c r="H114" s="44" t="inlineStr">
         <is>
           <t>Bonus attesi / punti di forza</t>
         </is>
       </c>
-      <c r="I113" s="44" t="inlineStr">
+      <c r="I114" s="44" t="inlineStr">
         <is>
           <t>Prezzo max</t>
         </is>
       </c>
-      <c r="J113" s="44" t="inlineStr">
+      <c r="J114" s="44" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>Hien</t>
-        </is>
-      </c>
-      <c r="C114" s="35" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="D114" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E114" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="F114" s="35" t="inlineStr">
-        <is>
-          <t>Rientro ottobre</t>
-        </is>
-      </c>
-      <c r="G114" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H114" s="36" t="inlineStr">
-        <is>
-          <t>Top a regime</t>
-        </is>
-      </c>
-      <c r="I114" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J114" s="36" t="inlineStr">
-        <is>
-          <t>Rientro post-sosta di settembre (~6ª), un filo prima del previsto. MA al rientro il posto non è garantito (titolari Kristensen e Scalvini): parcheggio a 1</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>Buongiorno</t>
+          <t>Hien</t>
         </is>
       </c>
       <c r="C115" s="35" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D115" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E115" s="10" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F115" s="35" t="inlineStr">
         <is>
-          <t>Rientro dic-gen?</t>
+          <t>Rientro ottobre</t>
         </is>
       </c>
       <c r="G115" s="35" t="inlineStr">
@@ -10060,33 +10104,33 @@
       </c>
       <c r="J115" s="36" t="inlineStr">
         <is>
-          <t>In dubbio fino alla ~12ª (radice menisco): peggio di Hien. Solo a 1 sapendo che è mezzo girone</t>
+          <t>Rientro post-sosta di settembre (~6ª), un filo prima del previsto. MA al rientro il posto non è garantito (titolari Kristensen e Scalvini): parcheggio a 1</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>Biraghi</t>
+          <t>Buongiorno</t>
         </is>
       </c>
       <c r="C116" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D116" s="10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E116" s="10" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="F116" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Rientro dic-gen?</t>
         </is>
       </c>
       <c r="G116" s="35" t="inlineStr">
@@ -10096,85 +10140,85 @@
       </c>
       <c r="H116" s="36" t="inlineStr">
         <is>
-          <t>Piazzati</t>
+          <t>Top a regime</t>
         </is>
       </c>
       <c r="I116" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J116" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come D7</t>
+          <t>In dubbio fino alla ~12ª (radice menisco): peggio di Hien. Solo a 1 sapendo che è mezzo girone</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Biraghi</t>
+        </is>
+      </c>
+      <c r="C117" s="35" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E117" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F117" s="35" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G117" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H117" s="36" t="inlineStr">
+        <is>
+          <t>Piazzati</t>
+        </is>
+      </c>
+      <c r="I117" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Bracaglia</t>
-        </is>
-      </c>
-      <c r="C117" s="35" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="D117" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E117" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="F117" s="35" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G117" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H117" s="36" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="I117" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="J117" s="36" t="inlineStr">
         <is>
-          <t>Se non preso prima</t>
+          <t>Se non preso come D7</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Bracaglia</t>
+        </is>
+      </c>
+      <c r="C118" s="35" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>Marin R.</t>
-        </is>
-      </c>
-      <c r="C118" s="35" t="inlineStr">
-        <is>
-          <t>Napoli</t>
-        </is>
-      </c>
-      <c r="D118" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="E118" s="10" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F118" s="35" t="inlineStr">
         <is>
-          <t>Titolare per emergenza</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G118" s="35" t="inlineStr">
@@ -10184,41 +10228,41 @@
       </c>
       <c r="H118" s="36" t="inlineStr">
         <is>
-          <t>Titolare del Napoli fino a ottobre</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="I118" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J118" s="36" t="inlineStr">
         <is>
-          <t>Titolare d'emergenza MA Badiashile in CHIUSURA (visite 18/8): rischio concreto e imminente. 1-2 max</t>
+          <t>Se non preso prima</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Marcandalli</t>
+        </is>
+      </c>
+      <c r="C119" s="35" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>Calvani</t>
-        </is>
-      </c>
-      <c r="C119" s="35" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="D119" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="E119" s="10" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F119" s="35" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Titolare (campo 16/8)</t>
         </is>
       </c>
       <c r="G119" s="35" t="inlineStr">
@@ -10228,7 +10272,7 @@
       </c>
       <c r="H119" s="36" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>GOL di testa su corner con l'Ascoli</t>
         </is>
       </c>
       <c r="I119" s="10" t="n">
@@ -10236,33 +10280,33 @@
       </c>
       <c r="J119" s="36" t="inlineStr">
         <is>
-          <t>Scommessa a 1-2</t>
+          <t>Braccetto titolare nel 3-4-2-1 di De Rossi; le guide lo citano solo come backup</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>Perez M.</t>
+          <t>Comuzzo</t>
         </is>
       </c>
       <c r="C120" s="35" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D120" s="10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E120" s="10" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F120" s="35" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Titolare di Abate (tibia da verificare)</t>
         </is>
       </c>
       <c r="G120" s="35" t="inlineStr">
@@ -10272,41 +10316,41 @@
       </c>
       <c r="H120" s="36" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Perno del terzetto granata</t>
         </is>
       </c>
       <c r="I120" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J120" s="36" t="inlineStr">
         <is>
-          <t>Tappabuchi</t>
+          <t>Uscito al 67' in Coppa (colpo tibia), indicazioni rassicuranti ma esami NON pubblicati. Bruciato (TuttoFantacalcio/BetFlag)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Mangas</t>
+          <t>Marin R.</t>
         </is>
       </c>
       <c r="C121" s="35" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D121" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E121" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="E121" s="10" t="n">
-        <v>15</v>
-      </c>
       <c r="F121" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>NON prendere (Badiashile in arrivo)</t>
         </is>
       </c>
       <c r="G121" s="35" t="inlineStr">
@@ -10316,41 +10360,41 @@
       </c>
       <c r="H121" s="36" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Titolare del Napoli fino a ottobre</t>
         </is>
       </c>
       <c r="I121" s="10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J121" s="36" t="inlineStr">
         <is>
-          <t>Se non preso prima. Titolare in Coppa ma bruciato: budget su.</t>
+          <t>Visite Badiashile martedì 18/8 a Villa Stuart, accordo totale: Marin 'destinato a salutare' (CdS)</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Mitaj</t>
+          <t>Calvani</t>
         </is>
       </c>
       <c r="C122" s="35" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D122" s="10" t="n">
         <v>4</v>
       </c>
       <c r="E122" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F122" s="35" t="inlineStr">
         <is>
-          <t>Titolare (campo 16/8)</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G122" s="35" t="inlineStr">
@@ -10360,41 +10404,41 @@
       </c>
       <c r="H122" s="36" t="inlineStr">
         <is>
-          <t>Quinto sinistro nuovo di De Rossi</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="I122" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J122" s="36" t="inlineStr">
         <is>
-          <t>RISOLTO: titolare nel 3-5-2 con l'Ascoli. Bruciato (FantaMaster/Goal): da 3 a 4-5</t>
+          <t>Scommessa a 1-2</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>Marusic</t>
+          <t>Perez M.</t>
         </is>
       </c>
       <c r="C123" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D123" s="10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E123" s="10" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F123" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G123" s="35" t="inlineStr">
@@ -10404,41 +10448,41 @@
       </c>
       <c r="H123" s="36" t="inlineStr">
         <is>
-          <t>Usato sicuro sulle fasce</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="I123" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J123" s="36" t="inlineStr">
         <is>
-          <t>Scommessa citata dalle guide: esperienza e titolarità nella Lazio</t>
+          <t>Tappabuchi</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>Kempf</t>
+          <t>Mangas</t>
         </is>
       </c>
       <c r="C124" s="35" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D124" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E124" s="10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F124" s="35" t="inlineStr">
         <is>
-          <t>Fuori dall'XI atteso</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G124" s="35" t="inlineStr">
@@ -10448,41 +10492,41 @@
       </c>
       <c r="H124" s="36" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="I124" s="10" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J124" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO: l'XI atteso del Como dà Chalobah-Ramon centrali. Solo a 1-2 da copertura.</t>
+          <t>Se non preso prima. Titolare in Coppa ma bruciato: budget su.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="16" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>Tavares N.</t>
+          <t>Mitaj</t>
         </is>
       </c>
       <c r="C125" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D125" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E125" s="10" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F125" s="35" t="inlineStr">
         <is>
-          <t>Ko ginocchio + ipotesi scambio</t>
+          <t>Titolare (campo 16/8)</t>
         </is>
       </c>
       <c r="G125" s="35" t="inlineStr">
@@ -10492,7 +10536,7 @@
       </c>
       <c r="H125" s="36" t="inlineStr">
         <is>
-          <t>Assist</t>
+          <t>Quinto sinistro nuovo di De Rossi</t>
         </is>
       </c>
       <c r="I125" s="10" t="n">
@@ -10500,49 +10544,181 @@
       </c>
       <c r="J125" s="36" t="inlineStr">
         <is>
-          <t>Infiammazione al ginocchio (fuori in Coppa, Pedraza titolare) e ipotesi scambio con Tomori: solo a saldo estremo.</t>
+          <t>RISOLTO: titolare nel 3-5-2 con l'Ascoli. Bruciato (FantaMaster/Goal): da 3 a 4-5</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Marusic</t>
+        </is>
+      </c>
+      <c r="C126" s="35" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E126" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F126" s="35" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G126" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H126" s="36" t="inlineStr">
+        <is>
+          <t>Usato sicuro sulle fasce</t>
+        </is>
+      </c>
+      <c r="I126" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J126" s="36" t="inlineStr">
+        <is>
+          <t>Scommessa citata dalle guide: esperienza e titolarità nella Lazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B126" s="5" t="inlineStr">
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Kempf</t>
+        </is>
+      </c>
+      <c r="C127" s="35" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E127" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="F127" s="35" t="inlineStr">
+        <is>
+          <t>Fuori dall'XI atteso</t>
+        </is>
+      </c>
+      <c r="G127" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H127" s="36" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J127" s="36" t="inlineStr">
+        <is>
+          <t>DECLASSATO: l'XI atteso del Como dà Chalobah-Ramon centrali. Solo a 1-2 da copertura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Tavares N.</t>
+        </is>
+      </c>
+      <c r="C128" s="35" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E128" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="F128" s="35" t="inlineStr">
+        <is>
+          <t>Ko ginocchio + ipotesi scambio</t>
+        </is>
+      </c>
+      <c r="G128" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H128" s="36" t="inlineStr">
+        <is>
+          <t>Assist</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J128" s="36" t="inlineStr">
+        <is>
+          <t>Infiammazione al ginocchio (fuori in Coppa, Pedraza titolare) e ipotesi scambio con Tomori: solo a saldo estremo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
         <is>
           <t>Correia T.</t>
         </is>
       </c>
-      <c r="C126" s="35" t="inlineStr">
+      <c r="C129" s="35" t="inlineStr">
         <is>
           <t>Venezia</t>
         </is>
       </c>
-      <c r="D126" s="10" t="n">
+      <c r="D129" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E126" s="10" t="n">
+      <c r="E129" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="F126" s="35" t="inlineStr">
+      <c r="F129" s="35" t="inlineStr">
         <is>
           <t>Superato da Hainaut</t>
         </is>
       </c>
-      <c r="G126" s="35" t="inlineStr">
+      <c r="G129" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H126" s="36" t="inlineStr">
+      <c r="H129" s="36" t="inlineStr">
         <is>
           <t>Venezia</t>
         </is>
       </c>
-      <c r="I126" s="10" t="n">
+      <c r="I129" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="J126" s="36" t="inlineStr">
+      <c r="J129" s="36" t="inlineStr">
         <is>
           <t>DECLASSATO DAL CAMPO: Hainaut titolare in Coppa, lui dentro al 74'. Solo ultimo slot.</t>
         </is>
@@ -10550,14 +10726,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A62:J62"/>
+    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A92:J92"/>
-    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A112:J112"/>
+    <mergeCell ref="A113:J113"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -10570,7 +10746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10597,7 +10773,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -10697,7 +10872,7 @@
       </c>
       <c r="J6" s="36" t="inlineStr">
         <is>
-          <t>BLINDATO sull'anno (Real ha rinunciato al riacquisto) MA cautela avvio: zero amichevoli post-Mondiale, titolare alla 1ª ~75%, e il Como in Champions ruoterà. Punizioni e corner suoi</t>
+          <t>Ha giocato 20' col Liverpool ('ha acceso la squadra') ma resta fuori dall'XI proiettato: alla 1ª ~60-75% con rischio spezzone. Sull'anno resta il C1 designato</t>
         </is>
       </c>
     </row>
@@ -11141,7 +11316,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -11311,7 +11485,7 @@
       </c>
       <c r="F22" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Risalito (~55%: provato da play)</t>
         </is>
       </c>
       <c r="G22" s="35" t="inlineStr">
@@ -11329,7 +11503,7 @@
       </c>
       <c r="J22" s="36" t="inlineStr">
         <is>
-          <t>Rigori+punizioni+corner e 1 solo giallo (fairplay top) MA fantacalcio.it 14/8 schiera Anguissa: minutaggio vero tema. Semi-top, non 1° slot.</t>
+          <t>Allegri lo prova REGISTA accanto a Lobotka: rientra nell'XI atteso. Rigorista 1° (5 fonti su 6) e 1° piazzati. Comprabile a prezzo medio, non più solo a sconto pieno</t>
         </is>
       </c>
     </row>
@@ -11685,7 +11859,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
@@ -11767,7 +11940,7 @@
       </c>
       <c r="F34" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Risalito (~55%: provato da play)</t>
         </is>
       </c>
       <c r="G34" s="35" t="inlineStr">
@@ -11785,7 +11958,7 @@
       </c>
       <c r="J34" s="36" t="inlineStr">
         <is>
-          <t>RAFFREDDATO: l'XI atteso (probabili + DAZN 15/8) dà la mediana Anguissa-Lobotka-McTominay con KDB fuori (30-45%). Rigori e piazzati confermati: solo a sconto pieno 25-35, non da semi-top</t>
+          <t>Allegri lo prova REGISTA accanto a Lobotka: rientra nell'XI atteso. Rigorista 1° e 1° piazzati. Comprabile a prezzo medio</t>
         </is>
       </c>
     </row>
@@ -12075,7 +12248,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>APERTO (tipo vs campo)</t>
+          <t>Panchina in Coppa (35% dal 1')</t>
         </is>
       </c>
       <c r="G41" s="35" t="inlineStr">
@@ -12089,7 +12262,7 @@
         </is>
       </c>
       <c r="I41" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J41" s="36" t="inlineStr">
         <is>
@@ -12229,7 +12402,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
@@ -12487,7 +12659,7 @@
       </c>
       <c r="F52" s="35" t="inlineStr">
         <is>
-          <t>Titolare (Gattuso)</t>
+          <t>Panchina anche col Mantova (dentro 70')</t>
         </is>
       </c>
       <c r="G52" s="35" t="inlineStr">
@@ -12501,11 +12673,11 @@
         </is>
       </c>
       <c r="I52" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J52" s="36" t="inlineStr">
         <is>
-          <t>UFFICIALE: titolare atteso col Bologna ma panchina al debutto di Coppa. Investimento, non low cost</t>
+          <t>50/50 con Dele-Bashiru alla 1ª + clima Lazio pessimo (eliminata, Gattuso contestato): l'investimento da 18 non è più giustificato</t>
         </is>
       </c>
     </row>
@@ -12751,7 +12923,7 @@
       </c>
       <c r="F58" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Titolare e in GOL il 16/8</t>
         </is>
       </c>
       <c r="G58" s="35" t="inlineStr">
@@ -12765,11 +12937,11 @@
         </is>
       </c>
       <c r="I58" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J58" s="36" t="inlineStr">
         <is>
-          <t>Titolare nella probabile di Coppa, 1° sulle punizioni: confermato ma bruciato.</t>
+          <t>Trequartista nel 3-4-2-1, gol all'Ascoli, 1° sulle punizioni. Bruciato: costerà</t>
         </is>
       </c>
     </row>
@@ -12817,7 +12989,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
@@ -13075,7 +13246,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Rowe nettamente favorito</t>
         </is>
       </c>
       <c r="G67" s="35" t="inlineStr">
@@ -13089,11 +13260,11 @@
         </is>
       </c>
       <c r="I67" s="10" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J67" s="36" t="inlineStr">
         <is>
-          <t>RIBALTATO IN MEGLIO: titolare a sinistra col Brighton, Rowe entrato a destra per Orsolini (55/45 pro Cambiaghi). Col cambio ruolo A→C torna un buon C5 a 4-6</t>
+          <t>BOCCIATO dalle probabili aggiornate: il segnale del Brighton non regge</t>
         </is>
       </c>
     </row>
@@ -13361,7 +13532,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -13751,7 +13921,7 @@
       </c>
       <c r="F84" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>INFORTUNATO (non convocato)</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -13765,11 +13935,11 @@
         </is>
       </c>
       <c r="I84" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J84" s="36" t="inlineStr">
         <is>
-          <t>Il faro del Lecce: potrebbe battere anche i rigori</t>
+          <t>Fuori per infortunio col Palermo e fuori dalla corsa rigori; i piazzati passano a Pierotti/Gandelman</t>
         </is>
       </c>
     </row>
@@ -13905,7 +14075,6 @@
         </is>
       </c>
     </row>
-    <row r="88"/>
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
         <is>
@@ -13992,7 +14161,7 @@
       </c>
       <c r="G91" s="35" t="inlineStr">
         <is>
-          <t>Sì (5/5 in B)</t>
+          <t>Sì (1° confermato da 4 fonti + tutti i piazzati)</t>
         </is>
       </c>
       <c r="H91" s="36" t="inlineStr">
@@ -14005,7 +14174,7 @@
       </c>
       <c r="J91" s="36" t="inlineStr">
         <is>
-          <t>Rigorista confermato da 7 fonti su 8 (outlier FantaMaster: Schmid); titolare nel 3-0 del 16/8 con tutti i piazzati. La certezza low cost del reparto</t>
+          <t>ATTENZIONE PREZZO: è ormai il rigorista low-cost più consigliato d'Italia (5+ fonti tra cui Goal a 1cr e BetFlag 5cr): comprarlo presto o pagarlo</t>
         </is>
       </c>
     </row>
@@ -14031,7 +14200,7 @@
       </c>
       <c r="F92" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>INFORTUNATO (non convocato)</t>
         </is>
       </c>
       <c r="G92" s="35" t="inlineStr">
@@ -14045,11 +14214,11 @@
         </is>
       </c>
       <c r="I92" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J92" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C6</t>
+          <t>Fuori per infortunio col Palermo; i piazzati passano a Pierotti/Gandelman</t>
         </is>
       </c>
     </row>
@@ -14427,7 +14596,7 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Riaperto (tipo)</t>
+          <t>Titolare (campo 15/8) ma bruciato</t>
         </is>
       </c>
       <c r="G101" s="35" t="inlineStr">
@@ -14441,15 +14610,14 @@
         </is>
       </c>
       <c r="I101" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J101" s="36" t="inlineStr">
         <is>
-          <t>RISOLTO: assenza per la nascita del figlio (falso allarme, il caso-mercato è Duncan). Titolare 45-55 col Lecce: a 1-2 free roll vero</t>
-        </is>
-      </c>
-    </row>
-    <row r="102"/>
+          <t>Falso allarme chiuso; Goal 'titolare garantito' e Lottomatica lo dà 1° punizioni (per noi 1° è Busio): prezzo su</t>
+        </is>
+      </c>
+    </row>
     <row r="103" ht="28" customHeight="1">
       <c r="A103" s="1" t="inlineStr">
         <is>
@@ -14531,7 +14699,7 @@
       </c>
       <c r="F105" s="35" t="inlineStr">
         <is>
-          <t>Titolare/capitano</t>
+          <t>Backup di Adopo (DAZN)</t>
         </is>
       </c>
       <c r="G105" s="35" t="inlineStr">
@@ -14545,11 +14713,11 @@
         </is>
       </c>
       <c r="I105" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J105" s="36" t="inlineStr">
         <is>
-          <t>Rigore VERO il 14/8 ma Pisacane frena ('c'è una gerarchia') e nessuna testata lo dà 1°; per DAZN non è nemmeno titolare fisso. Scommessa da 3-6, non di più</t>
+          <t>Nessuna lista rigori fresca lo cita (TuttoFantacalcio: Fazzini-Mina-Maldini). Il rigore di Coppa resta un episodio: 3-4 max</t>
         </is>
       </c>
     </row>
@@ -14735,7 +14903,7 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Fini</t>
+          <t>Cichella</t>
         </is>
       </c>
       <c r="C110" s="35" t="inlineStr">
@@ -14744,32 +14912,32 @@
         </is>
       </c>
       <c r="D110" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E110" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F110" s="35" t="inlineStr">
+        <is>
+          <t>Titolare e GOL il 16/8</t>
+        </is>
+      </c>
+      <c r="G110" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H110" s="36" t="inlineStr">
+        <is>
+          <t>Mediana titolare con Calò</t>
+        </is>
+      </c>
+      <c r="I110" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E110" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="F110" s="35" t="inlineStr">
-        <is>
-          <t>Assente il 16/8 (squalifica)</t>
-        </is>
-      </c>
-      <c r="G110" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H110" s="36" t="inlineStr">
-        <is>
-          <t>Tridente Frosinone dal campo</t>
-        </is>
-      </c>
-      <c r="I110" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="J110" s="36" t="inlineStr">
         <is>
-          <t>CORREZIONE: era squalificato, non bocciato. Ballottaggio esterno vivo dal rientro: 1-2</t>
+          <t>ZERO citazioni in tutte le guide: lo sleeper C più pulito insieme a Schmid</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14947,7 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Calò</t>
+          <t>Fini</t>
         </is>
       </c>
       <c r="C111" s="35" t="inlineStr">
@@ -14788,14 +14956,14 @@
         </is>
       </c>
       <c r="D111" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E111" s="10" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F111" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Rientra: 40/60 con Ghedjemis</t>
         </is>
       </c>
       <c r="G111" s="35" t="inlineStr">
@@ -14805,15 +14973,15 @@
       </c>
       <c r="H111" s="36" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Tridente Frosinone dal campo</t>
         </is>
       </c>
       <c r="I111" s="10" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="J111" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>Era squalificato in Coppa; dal rientro si gioca l'esterno (Ghedjemis avanti 60/40)</t>
         </is>
       </c>
     </row>
@@ -14823,23 +14991,23 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Perez K.</t>
+          <t>Calò</t>
         </is>
       </c>
       <c r="C112" s="35" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D112" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E112" s="10" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F112" s="35" t="inlineStr">
         <is>
-          <t>Titolare (campo)</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G112" s="35" t="inlineStr">
@@ -14849,15 +15017,15 @@
       </c>
       <c r="H112" s="36" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="I112" s="10" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="J112" s="36" t="inlineStr">
         <is>
-          <t>Piazzati del Venezia in canna: da ultimo slot è oro (ballottaggio con Sohm).</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -14867,12 +15035,12 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>Adzic</t>
+          <t>Perez K.</t>
         </is>
       </c>
       <c r="C113" s="35" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D113" s="10" t="n">
@@ -14883,7 +15051,7 @@
       </c>
       <c r="F113" s="35" t="inlineStr">
         <is>
-          <t>Titolare (55/45)</t>
+          <t>Titolare (campo)</t>
         </is>
       </c>
       <c r="G113" s="35" t="inlineStr">
@@ -14893,15 +15061,15 @@
       </c>
       <c r="H113" s="36" t="inlineStr">
         <is>
-          <t>2° tiratore di punizioni e corner dietro Berardi</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="I113" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J113" s="36" t="inlineStr">
         <is>
-          <t>APERTO: in Coppa atteso/impiegato Lipani, ma fantacalcio.it dà Adzic titolare alla 1ª: 50/50 vero.</t>
+          <t>Piazzati del Venezia in canna: da ultimo slot è oro (ballottaggio con Sohm).</t>
         </is>
       </c>
     </row>
@@ -14911,23 +15079,23 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Vergara</t>
+          <t>Adzic</t>
         </is>
       </c>
       <c r="C114" s="35" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D114" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E114" s="10" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="F114" s="35" t="inlineStr">
         <is>
-          <t>Recuperato</t>
+          <t>Titolare (55/45)</t>
         </is>
       </c>
       <c r="G114" s="35" t="inlineStr">
@@ -14937,15 +15105,15 @@
       </c>
       <c r="H114" s="36" t="inlineStr">
         <is>
-          <t>Gol in Champions, corner in rotazione</t>
+          <t>2° tiratore di punizioni e corner dietro Berardi</t>
         </is>
       </c>
       <c r="I114" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J114" s="36" t="inlineStr">
         <is>
-          <t>Rientrato in gruppo: la scommessa a 1-2 torna valida.</t>
+          <t>APERTO: in Coppa atteso/impiegato Lipani, ma fantacalcio.it dà Adzic titolare alla 1ª: 50/50 vero.</t>
         </is>
       </c>
     </row>
@@ -14955,23 +15123,23 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>Oristanio</t>
+          <t>Vergara</t>
         </is>
       </c>
       <c r="C115" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D115" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E115" s="10" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F115" s="35" t="inlineStr">
         <is>
-          <t>Riaperto (tipo)</t>
+          <t>Recuperato</t>
         </is>
       </c>
       <c r="G115" s="35" t="inlineStr">
@@ -14981,15 +15149,15 @@
       </c>
       <c r="H115" s="36" t="inlineStr">
         <is>
-          <t>2° tiratore piazzati dietro Vlasic</t>
+          <t>Gol in Champions, corner in rotazione</t>
         </is>
       </c>
       <c r="I115" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J115" s="36" t="inlineStr">
         <is>
-          <t>CONFLITTO: panchina in Coppa il 15/8 MA trequartista titolare nella formazione-tipo di Abate. 50/50 vero con Casadei: a 2-3 ci sta di nuovo</t>
+          <t>Rientrato in gruppo: la scommessa a 1-2 torna valida.</t>
         </is>
       </c>
     </row>
@@ -14999,23 +15167,23 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>Milla</t>
+          <t>Oristanio</t>
         </is>
       </c>
       <c r="C116" s="35" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D116" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E116" s="10" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F116" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Panchina in Coppa + bruciato</t>
         </is>
       </c>
       <c r="G116" s="35" t="inlineStr">
@@ -15025,15 +15193,15 @@
       </c>
       <c r="H116" s="36" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>2° tiratore piazzati dietro Vlasic</t>
         </is>
       </c>
       <c r="I116" s="10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J116" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>CONFLITTO: panchina in Coppa il 15/8 MA trequartista titolare nella formazione-tipo di Abate. 50/50 vero con Casadei: a 2-3 ci sta di nuovo</t>
         </is>
       </c>
     </row>
@@ -15043,41 +15211,41 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>Colpani</t>
+          <t>Milla</t>
         </is>
       </c>
       <c r="C117" s="35" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D117" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E117" s="10" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F117" s="35" t="inlineStr">
         <is>
-          <t>Titolare (tipo)</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G117" s="35" t="inlineStr">
         <is>
-          <t>Outsider (2° pre-infortunio Pessina)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H117" s="36" t="inlineStr">
         <is>
-          <t>Punizioni e corner del Monza</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="I117" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J117" s="36" t="inlineStr">
         <is>
-          <t>Con Pessina out fino a novembre è l'outsider-rigori (Sky lo dava 2°) e batte i piazzati; entrato al 70' in Coppa. Nessuno lo prezza per questo</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -15087,41 +15255,41 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>Aboukhlal</t>
+          <t>Colpani</t>
         </is>
       </c>
       <c r="C118" s="35" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D118" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E118" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F118" s="35" t="inlineStr">
+        <is>
+          <t>Titolare ~60% (panchina in Coppa)</t>
+        </is>
+      </c>
+      <c r="G118" s="35" t="inlineStr">
+        <is>
+          <t>Outsider (punizioni sue con Pessina out)</t>
+        </is>
+      </c>
+      <c r="H118" s="36" t="inlineStr">
+        <is>
+          <t>Punizioni e corner del Monza</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="F118" s="35" t="inlineStr">
-        <is>
-          <t>Fondo gerarchie</t>
-        </is>
-      </c>
-      <c r="G118" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H118" s="36" t="inlineStr">
-        <is>
-          <t>Cambio ruolo A→C</t>
-        </is>
-      </c>
-      <c r="I118" s="10" t="n">
-        <v>1</v>
-      </c>
       <c r="J118" s="36" t="inlineStr">
         <is>
-          <t>SMENTITO dalle probabili: nessuna fonte lo dà titolare (DAZN lo mette dietro Vlasic/Oristanio/Njie). Solo ultimo slot a 1.</t>
+          <t>Cutrone 1° fino a novembre; Colpani batte punizioni/corner ma in Coppa è partito fuori (Forson l'emergente in gol)</t>
         </is>
       </c>
     </row>
@@ -15131,23 +15299,23 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>Busio</t>
+          <t>Aboukhlal</t>
         </is>
       </c>
       <c r="C119" s="35" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D119" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E119" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="E119" s="10" t="n">
-        <v>14</v>
-      </c>
       <c r="F119" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Fondo gerarchie</t>
         </is>
       </c>
       <c r="G119" s="35" t="inlineStr">
@@ -15157,15 +15325,15 @@
       </c>
       <c r="H119" s="36" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Cambio ruolo A→C</t>
         </is>
       </c>
       <c r="I119" s="10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J119" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C7</t>
+          <t>SMENTITO dalle probabili: nessuna fonte lo dà titolare (DAZN lo mette dietro Vlasic/Oristanio/Njie). Solo ultimo slot a 1.</t>
         </is>
       </c>
     </row>
@@ -15175,23 +15343,23 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>Zhegrova</t>
+          <t>Busio</t>
         </is>
       </c>
       <c r="C120" s="35" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D120" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E120" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F120" s="35" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Altissima</t>
         </is>
       </c>
       <c r="G120" s="35" t="inlineStr">
@@ -15201,15 +15369,15 @@
       </c>
       <c r="H120" s="36" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="I120" s="10" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J120" s="36" t="inlineStr">
         <is>
-          <t>Se non preso come C5</t>
+          <t>Se non preso come C7</t>
         </is>
       </c>
     </row>
@@ -15219,23 +15387,23 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Isaksen</t>
+          <t>Zhegrova</t>
         </is>
       </c>
       <c r="C121" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D121" s="10" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E121" s="10" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F121" s="35" t="inlineStr">
         <is>
-          <t>Alta (post-infortunio)</t>
+          <t>Ballottaggio</t>
         </is>
       </c>
       <c r="G121" s="35" t="inlineStr">
@@ -15245,15 +15413,15 @@
       </c>
       <c r="H121" s="36" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="I121" s="10" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J121" s="36" t="inlineStr">
         <is>
-          <t>Scommessa di lusso se il prezzo crolla</t>
+          <t>Se non preso come C5</t>
         </is>
       </c>
     </row>
@@ -15263,23 +15431,23 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Stankovic A.</t>
+          <t>Isaksen</t>
         </is>
       </c>
       <c r="C122" s="35" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D122" s="10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E122" s="10" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F122" s="35" t="inlineStr">
         <is>
-          <t>Bassa</t>
+          <t>Alta (post-infortunio)</t>
         </is>
       </c>
       <c r="G122" s="35" t="inlineStr">
@@ -15289,15 +15457,15 @@
       </c>
       <c r="H122" s="36" t="inlineStr">
         <is>
-          <t>Talento Inter</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="I122" s="10" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="J122" s="36" t="inlineStr">
         <is>
-          <t>Puro parcheggio a 1: minutaggio da verificare</t>
+          <t>Scommessa di lusso se il prezzo crolla</t>
         </is>
       </c>
     </row>
@@ -15307,23 +15475,23 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Stankovic A.</t>
         </is>
       </c>
       <c r="C123" s="35" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="D123" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E123" s="10" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F123" s="35" t="inlineStr">
         <is>
-          <t>CONGELATO</t>
+          <t>Bassa</t>
         </is>
       </c>
       <c r="G123" s="35" t="inlineStr">
@@ -15333,7 +15501,7 @@
       </c>
       <c r="H123" s="36" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Talento Inter</t>
         </is>
       </c>
       <c r="I123" s="10" t="n">
@@ -15341,20 +15509,64 @@
       </c>
       <c r="J123" s="36" t="inlineStr">
         <is>
+          <t>Puro parcheggio a 1: minutaggio da verificare</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="C124" s="35" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E124" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="F124" s="35" t="inlineStr">
+        <is>
+          <t>Titolare (campo 15/8) ma bruciato</t>
+        </is>
+      </c>
+      <c r="G124" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H124" s="36" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J124" s="36" t="inlineStr">
+        <is>
           <t>Dato titolare alla vigilia, poi né in campo né tra i subentrati in Coppa (possibile mercato): congelare.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A103:J103"/>
+    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A32:J32"/>
-    <mergeCell ref="A75:J75"/>
-    <mergeCell ref="A89:J89"/>
     <mergeCell ref="A61:J61"/>
     <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A89:J89"/>
+    <mergeCell ref="A103:J103"/>
     <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A75:J75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -15367,7 +15579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15493,7 +15705,7 @@
       </c>
       <c r="J6" s="36" t="inlineStr">
         <is>
-          <t>AVVIO A RISCHIO CONFERMATO da 2 filoni: 45% titolare alla 1ª (Bonny 80, Esposito 60, Thuram 20). Profilo A1 intatto sull'anno; sopra ~200 il margine sparisce</t>
+          <t>Alla 1ª ~25% (condizione indietro, panchina col Betis). Profilo A1 intatto sull'anno: sfruttare lo sconto d'avvio</t>
         </is>
       </c>
     </row>
@@ -15563,7 +15775,7 @@
       </c>
       <c r="F8" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Altissima sull'anno; 1ª a rischio (15-20%)</t>
         </is>
       </c>
       <c r="G8" s="35" t="inlineStr">
@@ -15581,7 +15793,7 @@
       </c>
       <c r="J8" s="36" t="inlineStr">
         <is>
-          <t>Polpaccio: rimasto ad Appiano anche col Betis; titolare alla 1ª solo se risolve tutto. fantacalcio.it (80%) è in ritardo: sconto d'avvio</t>
+          <t>Polpaccio + Chivu: 'ne dubito' sui titolari. Alla 1ª col Monza favoriti Bonny-Esposito</t>
         </is>
       </c>
     </row>
@@ -15757,7 +15969,7 @@
       </c>
       <c r="J12" s="36" t="inlineStr">
         <is>
-          <t>Ci aspettiamo il suo totale riscatto in viola</t>
+          <t>ASSALTO COMO IN CORSO: rilancio atteso a ore (TMW 17/8), 35-45M sul piatto; la Fiorentina chiede 45-50 e dice di tenerlo. Prezzare il rischio fino all'1/9</t>
         </is>
       </c>
     </row>
@@ -16080,7 +16292,7 @@
       </c>
       <c r="J21" s="36" t="inlineStr">
         <is>
-          <t>Punta unica confermata al 90/10 (Pellegrino arriva da vice e alla 1ª è indisponibile): il posto è blindato. Rigori dietro Gudmundsson.</t>
+          <t>ASSALTO COMO IN CORSO: rilancio atteso a ore (TMW 17/8). Prezzare il rischio fino all'1/9</t>
         </is>
       </c>
     </row>
@@ -16414,12 +16626,12 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Preseason SALTATA: 1ª a rischio (35%)</t>
         </is>
       </c>
       <c r="G29" s="35" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>Sì sulla carta (Laurienté de facto all'avvio)</t>
         </is>
       </c>
       <c r="H29" s="36" t="inlineStr">
@@ -16428,11 +16640,11 @@
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="J29" s="36" t="inlineStr">
         <is>
-          <t>Non nelle tabelle infortunati (buon segno) ma non in gruppo pieno e fuori dalla probabile col Cesena: convocati del 17/8 decisivi. Scontare</t>
+          <t>Fermo da febbraio (caviglia), Aquilani: 'spero di riaverlo presto'; probabili di stasera discordanti. NON pagarlo da rigorista attivo</t>
         </is>
       </c>
     </row>
@@ -16693,12 +16905,12 @@
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Preseason SALTATA: 1ª a rischio (35%)</t>
         </is>
       </c>
       <c r="G37" s="35" t="inlineStr">
         <is>
-          <t>Sì</t>
+          <t>Sì sulla carta (Laurienté de facto all'avvio)</t>
         </is>
       </c>
       <c r="H37" s="36" t="inlineStr">
@@ -16707,11 +16919,11 @@
         </is>
       </c>
       <c r="I37" s="10" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="J37" s="36" t="inlineStr">
         <is>
-          <t>In dubbio per la 1ª (caviglia, programma personalizzato): scontare l'avvio.</t>
+          <t>Fermo da febbraio, probabili discordanti: non pagarlo da rigorista attivo</t>
         </is>
       </c>
     </row>
@@ -16737,7 +16949,7 @@
       </c>
       <c r="F38" s="35" t="inlineStr">
         <is>
-          <t>A rischio 1ª (adduttori)</t>
+          <t>OUT 1ª, rientro inizio settembre</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -16751,11 +16963,11 @@
         </is>
       </c>
       <c r="I38" s="10" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="J38" s="36" t="inlineStr">
         <is>
-          <t>OUT confermato per la 1ª (in dubbio anche 2ª). Due aggregatori lo schierano ancora: comprarlo con lo sconto-infortunio.</t>
+          <t>Peggiorato (dubbio anche 2ª). Nel tridente del 4-3-3 al rientro: comprare solo con sconto pieno</t>
         </is>
       </c>
     </row>
@@ -16825,7 +17037,7 @@
       </c>
       <c r="F40" s="35" t="inlineStr">
         <is>
-          <t>Titolare alla 1ª (60%)</t>
+          <t>Titolare alla 1ª (75%)</t>
         </is>
       </c>
       <c r="G40" s="35" t="inlineStr">
@@ -16843,7 +17055,7 @@
       </c>
       <c r="J40" s="36" t="inlineStr">
         <is>
-          <t>CAMBIATO IN MEGLIO: con Lautaro non in condizione parte TITOLARE (Bonny 80/Esposito 60/Lautaro 45): l'hype scontato ora è un'occasione d'avvio</t>
+          <t>XI col Betis: Bonny-Esposito. L'avvio è suo con Lautaro/Thuram indietro</t>
         </is>
       </c>
     </row>
@@ -16874,7 +17086,7 @@
       </c>
       <c r="G41" s="35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>De facto all'avvio (Berardi non pronto)</t>
         </is>
       </c>
       <c r="H41" s="36" t="inlineStr">
@@ -16883,11 +17095,11 @@
         </is>
       </c>
       <c r="I41" s="10" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J41" s="36" t="inlineStr">
         <is>
-          <t>Uno dei tre del Sassuolo che danno maggiori garanzie</t>
+          <t>Con Berardi fuori e Pinamonti sul mercato è lui il tiratore del Sassuolo</t>
         </is>
       </c>
     </row>
@@ -17153,7 +17365,7 @@
       </c>
       <c r="G49" s="35" t="inlineStr">
         <is>
-          <t>NO (nessun designato)</t>
+          <t>Candidato 1° (quadro conteso)</t>
         </is>
       </c>
       <c r="H49" s="36" t="inlineStr">
@@ -17162,11 +17374,11 @@
         </is>
       </c>
       <c r="I49" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J49" s="36" t="inlineStr">
         <is>
-          <t>RIDIMENSIONATO SUI RIGORI: titolare e assist in Coppa ma nessuno specialista designato nel Parma (Bernabè il candidato).</t>
+          <t>Post-Pellegrino: Goal 16/8 lo dà 1° (3/3); TuttoFantacalcio dà Valeri, F-online Bernabè. Premio-rigori piccolo. Occhio all'omonimo Idrissa Tourè (va al Monza)</t>
         </is>
       </c>
     </row>
@@ -17236,7 +17448,7 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Trattativa Lazio AVANZATA</t>
+          <t>Out per mercato: trattativa Lazio VIVA</t>
         </is>
       </c>
       <c r="G51" s="35" t="inlineStr">
@@ -17250,11 +17462,11 @@
         </is>
       </c>
       <c r="I51" s="10" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="J51" s="36" t="inlineStr">
         <is>
-          <t>FRENATO: budget Lazio 3-4M per due colpi + serve il rinnovo col Sassuolo; Icardi più compatibile. Resta out per mercato: non comprarlo da 9 titolare</t>
+          <t>CORREZIONE: non è ferma — Sassuolo chiede 15M, Lazio ~10M, nodo formula; ok del giocatore dato. Escluso col Cesena per tutela</t>
         </is>
       </c>
     </row>
@@ -17280,7 +17492,7 @@
       </c>
       <c r="F52" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Rottura totale col Cagliari: NON comprare</t>
         </is>
       </c>
       <c r="G52" s="35" t="inlineStr">
@@ -17294,11 +17506,11 @@
         </is>
       </c>
       <c r="I52" s="10" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="J52" s="36" t="inlineStr">
         <is>
-          <t>GUERRA col club: secondo certificato medico (altri 15 giorni), distanza Atalanta enorme. NON comprare.</t>
+          <t>Fuori dal progetto, stallo Como (10M+contropartite vs 20M cash), anche Napoli/Lazio alla finestra. Solo se si sblocca prima dell'asta</t>
         </is>
       </c>
     </row>
@@ -17324,7 +17536,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Assente in Coppa</t>
+          <t>In personalizzato: 1ª a rischio</t>
         </is>
       </c>
       <c r="G53" s="35" t="inlineStr">
@@ -17338,7 +17550,7 @@
         </is>
       </c>
       <c r="I53" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J53" s="36" t="inlineStr">
         <is>
@@ -17386,7 +17598,7 @@
       </c>
       <c r="J54" s="36" t="inlineStr">
         <is>
-          <t>L'agente tratta con Sunderland e Fulham (~35M): rischio-plusvalenza FFP tornato concreto (bookie 1,70 sull'addio). Sconto-mercato pieno</t>
+          <t>Doppio fronte: Sunderland/Fulham (nessuna offerta formale) + proposto al MILAN nell'ipotesi scambio con Nkunku. Sconto-mercato pieno fino all'1/9</t>
         </is>
       </c>
     </row>
@@ -17603,7 +17815,7 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>OUT 1ª (rientro col Torino)</t>
         </is>
       </c>
       <c r="G61" s="35" t="inlineStr">
@@ -17617,7 +17829,7 @@
         </is>
       </c>
       <c r="I61" s="10" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J61" s="36" t="inlineStr">
         <is>
@@ -17735,7 +17947,7 @@
       </c>
       <c r="F64" s="35" t="inlineStr">
         <is>
-          <t>Alta (rotazioni)</t>
+          <t>In pole alla 1ª (85%)</t>
         </is>
       </c>
       <c r="G64" s="35" t="inlineStr">
@@ -17749,11 +17961,11 @@
         </is>
       </c>
       <c r="I64" s="10" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J64" s="36" t="inlineStr">
         <is>
-          <t>UPGRADE AVVIO: 80% titolare alla 1ª con la ThuLa non al meglio. Il quarto slot d'avvio migliore del listone</t>
+          <t>XI col Betis con assist: con ThuLa indietro l'avvio è suo. 6-8 non bastano più</t>
         </is>
       </c>
     </row>
@@ -17779,7 +17991,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Altissima</t>
+          <t>Panchina col Palermo (XI probabile)</t>
         </is>
       </c>
       <c r="G65" s="35" t="inlineStr">
@@ -17797,7 +18009,7 @@
       </c>
       <c r="J65" s="36" t="inlineStr">
         <is>
-          <t>Alternativa nel tipo (posto a Geubbels) ma ha segnato un rigore in amichevole: contro-scommessa a 2-3</t>
+          <t>Geubbels titolare e 1° rigorista (5-3, 7/7 in carriera): contro-scommessa solo a 1-2</t>
         </is>
       </c>
     </row>
@@ -17955,7 +18167,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Ballottaggio</t>
+          <t>Titolare (65%: Pinamonti fuori per mercato)</t>
         </is>
       </c>
       <c r="G69" s="35" t="inlineStr">
@@ -17969,11 +18181,11 @@
         </is>
       </c>
       <c r="I69" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J69" s="36" t="inlineStr">
         <is>
-          <t>DECLASSATO: vice-Pinamonti (alternativa nel tipo), trigger-Lazio congelato dal budget. Scommessa condizionata a 4-6</t>
+          <t>RIALZATO: 9 titolare nelle probabili di stasera; se Pinamonti parte è il 9 del Sassuolo. Bruciato (FantaMaster/Goal)</t>
         </is>
       </c>
     </row>
@@ -18160,11 +18372,11 @@
         </is>
       </c>
       <c r="I75" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J75" s="36" t="inlineStr">
         <is>
-          <t>DOPPIETTA da titolare nel 3-0 del 16/8: domani è su tutte le guide. Alzare il tetto a 10-12 e comprarlo presto</t>
+          <t>BRUCIATO NELLE ULTIME ORE: doppietta su ANSA/Sportmediaset, Goal 1cr, FantaCalcioPedia 4-5cr. Comprarlo SUBITO o lasciar perdere: il prezzo sale stasera</t>
         </is>
       </c>
     </row>
@@ -18366,7 +18578,7 @@
       </c>
       <c r="F80" s="35" t="inlineStr">
         <is>
-          <t>FUORI dall'XI di Coppa</t>
+          <t>Titolare il 16/8 (uscito al 46')</t>
         </is>
       </c>
       <c r="G80" s="35" t="inlineStr">
@@ -18384,7 +18596,7 @@
       </c>
       <c r="J80" s="36" t="inlineStr">
         <is>
-          <t>Titolare nel tridente il 16/8 (allarme parzialmente rientrato) MA alternativa nel tipo e già bruciato: comprare a 2-4, non a 8</t>
+          <t>CORREZIONE: era nell'XI di Coppa. Dal rientro di Fini: 60/40. Bruciatissimo (TuttoFantacalcio 15cr!): 3-5 max</t>
         </is>
       </c>
     </row>
@@ -18575,7 +18787,7 @@
       </c>
       <c r="C85" s="35" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D85" s="10" t="n">
@@ -18586,7 +18798,7 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Alta (rotazioni)</t>
+          <t>Co-titolare (45/55 con Dovbyk)</t>
         </is>
       </c>
       <c r="G85" s="35" t="inlineStr">
@@ -18600,11 +18812,11 @@
         </is>
       </c>
       <c r="I85" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J85" s="36" t="inlineStr">
         <is>
-          <t>UFFICIALE al Bologna ma è il VICE-Dovbyk (30%), non trequartista: non pagarlo da titolare.</t>
+          <t>CORREZIONE SQUADRA: è al BOLOGNA (Qt 8), preso il 14/8 per duellare con Dovbyk; esordio già fatto col Brighton. Gli aggregatori non lo hanno ancora</t>
         </is>
       </c>
     </row>
@@ -18630,7 +18842,7 @@
       </c>
       <c r="F86" s="35" t="inlineStr">
         <is>
-          <t>Titolare col Mantova (16/8)</t>
+          <t>Subentro col Mantova (Dia titolare)</t>
         </is>
       </c>
       <c r="G86" s="35" t="inlineStr">
@@ -18644,7 +18856,7 @@
         </is>
       </c>
       <c r="I86" s="10" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J86" s="36" t="inlineStr">
         <is>
@@ -18674,7 +18886,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Forfait quasi certo (adduttore)</t>
+          <t>Ko all'intervallo il 14/8: forfait probabile</t>
         </is>
       </c>
       <c r="G87" s="35" t="inlineStr">
@@ -18688,11 +18900,11 @@
         </is>
       </c>
       <c r="I87" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J87" s="36" t="inlineStr">
         <is>
-          <t>Uscito all'intervallo per motivo medico, forfait quasi certo col Parma: scende a 1-2. Davanti ora c'è Borrelli (60-65%)</t>
+          <t>Era TITOLARE da 9 con l'Arezzo, poi distrazione adduttore: fonti sarde pessimiste, DAZN lo tiene 50/50. Se out: Borrelli</t>
         </is>
       </c>
     </row>
@@ -18702,41 +18914,41 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Ekhator</t>
+          <t>Borrelli</t>
         </is>
       </c>
       <c r="C88" s="35" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D88" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E88" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F88" s="35" t="inlineStr">
+        <is>
+          <t>9 atteso se Mendy non recupera</t>
+        </is>
+      </c>
+      <c r="G88" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H88" s="36" t="inlineStr">
+        <is>
+          <t>Subentrato in Coppa</t>
+        </is>
+      </c>
+      <c r="I88" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E88" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F88" s="35" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G88" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H88" s="36" t="inlineStr">
-        <is>
-          <t>Prospettiva Juve</t>
-        </is>
-      </c>
-      <c r="I88" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="J88" s="36" t="inlineStr">
         <is>
-          <t>Bicipite femorale ko, punta la 1ª: sorpresa da subentro dietro Kolo Muani (FantaMaster). Ultimo slot.</t>
+          <t>Con Mendy ko e Kevin Carlos in personalizzato è il candidato col Parma; bruciato (Goal/sportcafe24) e non certo</t>
         </is>
       </c>
     </row>
@@ -18746,23 +18958,23 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Noslin</t>
+          <t>Ekhator</t>
         </is>
       </c>
       <c r="C89" s="35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D89" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E89" s="10" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Titolare col Mantova (16/8)</t>
+          <t>Infortunato (lesione coscia)</t>
         </is>
       </c>
       <c r="G89" s="35" t="inlineStr">
@@ -18772,15 +18984,15 @@
       </c>
       <c r="H89" s="36" t="inlineStr">
         <is>
-          <t>Jolly offensivo Lazio</t>
+          <t>Prospettiva Juve</t>
         </is>
       </c>
       <c r="I89" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J89" s="36" t="inlineStr">
         <is>
-          <t>PROMOSSO: nel tridente titolare all'esordio di Gattuso con Zaccagni e Ratkov. La corsa a tre si è riaperta</t>
+          <t>Bicipite femorale ko, punta la 1ª: sorpresa da subentro dietro Kolo Muani (FantaMaster). Ultimo slot.</t>
         </is>
       </c>
     </row>
@@ -18790,39 +19002,127 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
+          <t>Havel</t>
+        </is>
+      </c>
+      <c r="C90" s="35" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E90" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F90" s="35" t="inlineStr">
+        <is>
+          <t>Prima alternativa a Colombo</t>
+        </is>
+      </c>
+      <c r="G90" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>GOL da subentrato il 16/8</t>
+        </is>
+      </c>
+      <c r="I90" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J90" s="36" t="inlineStr">
+        <is>
+          <t>Recuperato, convocato e subito in gol: scommessa da ultimo slot che nessuna guida cita</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Noslin</t>
+        </is>
+      </c>
+      <c r="C91" s="35" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E91" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="F91" s="35" t="inlineStr">
+        <is>
+          <t>Subentro col Mantova</t>
+        </is>
+      </c>
+      <c r="G91" s="35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" s="36" t="inlineStr">
+        <is>
+          <t>Jolly offensivo Lazio</t>
+        </is>
+      </c>
+      <c r="I91" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J91" s="36" t="inlineStr">
+        <is>
+          <t>PROMOSSO: nel tridente titolare all'esordio di Gattuso con Zaccagni e Ratkov. La corsa a tre si è riaperta</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
           <t>Varela G.</t>
         </is>
       </c>
-      <c r="C90" s="35" t="inlineStr">
+      <c r="C92" s="35" t="inlineStr">
         <is>
           <t>Monza</t>
         </is>
       </c>
-      <c r="D90" s="10" t="n">
+      <c r="D92" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E90" s="10" t="n">
+      <c r="E92" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="F90" s="35" t="inlineStr">
+      <c r="F92" s="35" t="inlineStr">
         <is>
           <t>Seconda punta (campo)</t>
         </is>
       </c>
-      <c r="G90" s="35" t="inlineStr">
+      <c r="G92" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H90" s="36" t="inlineStr">
+      <c r="H92" s="36" t="inlineStr">
         <is>
           <t>Doppietta in Coppa dietro Cutrone</t>
         </is>
       </c>
-      <c r="I90" s="10" t="n">
+      <c r="I92" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="J90" s="36" t="inlineStr">
+      <c r="J92" s="36" t="inlineStr">
         <is>
           <t>Doppietta da titolare il 14/8, zero copertura mediatica: ultimo slot con upside vero, target 4-5</t>
         </is>
@@ -18830,12 +19130,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A72:J72"/>
     <mergeCell ref="A45:J45"/>
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="A58:J58"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A72:J72"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>